<commit_message>
iGaming batch 01: 10 companies populated, calibration anchors set
First real output from the Opus->Sonnet orchestration loop. 10/10 companies
returned, QA-gated, written with computed scores.

- EPI range 26-76, all four quadrants represented, tiers 4 High / 3 Med / 3 Low
- Frame discipline holding: Bet365 is huge (D 94) but scores Sleeping giant
  (EPI 48) on low willingness, while DraftKings at D 70 scores higher (EPI 60).
  Betsson, the named incumbent, correctly lands low - it is the model being
  disrupted, not a disruptor.
- anchors.md records the scale for every future batch; qa_check.py now fails on
  >8 EPI points of anchor drift
- Documented one accepted deviation: Evolution researched to Dormant (26), not
  the Sleeping giant the seed list predicted - it has no player-facing rails
  under this frame, so the researched value wins

qa_check: 10 passed, 0 warnings, 0 failures.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/industries/igaming/igaming_landscape.xlsx
+++ b/industries/igaming/igaming_landscape.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DL3"/>
+  <dimension ref="A1:DL13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1292,6 +1292,3317 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Flutter Entertainment plc</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Dublin, Ireland (primary listing NYSE since 2024/25 redomicile)</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>2016</v>
+      </c>
+      <c r="F4" t="n">
+        <v>18130</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Operator (B2C)</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Multi-brand global sportsbook/casino operator (FanDuel US; Paddy Power, Betfair, Sky Bet UK; Sisal Italy; PokerStars; Junglee Games) monetizing GGR; expanding into CFTC-regulated prediction markets via the FanDuel Predicts joint venture with CME Group.</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>B2C — mass-market sports bettors and casino players across US, UK/Ireland, Italy, Australia, Brazil, India and other markets</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>Proprietary quant pricing/risk models, now commercialized to third parties; no evidence of frontier LLM training</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>15.9M average monthly players across a global multi-vertical footprint; proprietary pricing/risk tech now sold as a B2B service</t>
+        </is>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>CME Group (FanDuel Predicts JV)</t>
+        </is>
+      </c>
+      <c r="AH4" t="inlineStr">
+        <is>
+          <t>US (multi-state via FanDuel), UK, Ireland, Italy, Australia, Brazil, India, plus Malta/Gibraltar point-of-supply licences</t>
+        </is>
+      </c>
+      <c r="AK4" t="inlineStr">
+        <is>
+          <t>Standard safer-gambling tools (deposit/loss limits, self-exclusion) as a licence condition across brands; not independently verified this session</t>
+        </is>
+      </c>
+      <c r="AM4" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AN4" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AO4" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AP4" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AQ4" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AR4" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AS4" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AT4" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AV4" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AZ4" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="BB4" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="BD4" t="n">
+        <v>5</v>
+      </c>
+      <c r="BI4" t="n">
+        <v>4</v>
+      </c>
+      <c r="BJ4" t="n">
+        <v>4</v>
+      </c>
+      <c r="BK4" t="n">
+        <v>4</v>
+      </c>
+      <c r="BL4" t="n">
+        <v>5</v>
+      </c>
+      <c r="BM4" t="n">
+        <v>5</v>
+      </c>
+      <c r="BN4" t="n">
+        <v>5</v>
+      </c>
+      <c r="BO4" t="n">
+        <v>5</v>
+      </c>
+      <c r="BP4" t="n">
+        <v>5</v>
+      </c>
+      <c r="BQ4" t="n">
+        <v>3</v>
+      </c>
+      <c r="BR4" t="n">
+        <v>5</v>
+      </c>
+      <c r="BS4" t="n">
+        <v>5</v>
+      </c>
+      <c r="BT4" t="n">
+        <v>3</v>
+      </c>
+      <c r="BU4" t="n">
+        <v>1</v>
+      </c>
+      <c r="BV4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW4" t="n">
+        <v>2</v>
+      </c>
+      <c r="BX4" t="n">
+        <v>4</v>
+      </c>
+      <c r="BY4" t="n">
+        <v>5</v>
+      </c>
+      <c r="BZ4" t="n">
+        <v>3</v>
+      </c>
+      <c r="CA4" t="n">
+        <v>86</v>
+      </c>
+      <c r="CB4" t="n">
+        <v>94</v>
+      </c>
+      <c r="CC4" t="n">
+        <v>47</v>
+      </c>
+      <c r="CD4" t="n">
+        <v>70</v>
+      </c>
+      <c r="CE4" t="n">
+        <v>76</v>
+      </c>
+      <c r="CF4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="CG4" t="inlineStr">
+        <is>
+          <t>Imminent threat</t>
+        </is>
+      </c>
+      <c r="CH4" t="inlineStr">
+        <is>
+          <t>No shipped agentic/conversational betting assistant yet; still funds significant paid acquisition alongside owned app growth.</t>
+        </is>
+      </c>
+      <c r="CJ4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="CK4" t="inlineStr">
+        <is>
+          <t>0-12m</t>
+        </is>
+      </c>
+      <c r="CL4" t="inlineStr">
+        <is>
+          <t>As the largest incumbent operator itself, Flutter is racing to build the owned player-surface (FanDuel One App) that other operators must now match or fall behind.</t>
+        </is>
+      </c>
+      <c r="CN4" t="inlineStr">
+        <is>
+          <t>Legal entity Flutter Entertainment plc (NYSE primary listing, formerly Paddy Power Betfair plc, renamed 2019). FanDuel (US), Paddy Power, Betfair, Sky Bet (UK), Sisal (Italy), PokerStars, Junglee Games, Adjarabet and Betnacional are brands/subsidiaries, not separate legal entities — scored at Flutter parent level. FanDuel Predicts is a JV with CME Group, not wholly owned. Serves as one of the batch's calibration anchors (frame.md expected shape: high W, high D, high-mid AI -&gt; Imminent threat) — scores here effectively establish that anchor pending anchors.md.</t>
+        </is>
+      </c>
+      <c r="CQ4" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="CU4" t="inlineStr">
+        <is>
+          <t>$18.4B FY2025 revenue (+19% YoY), adjusted EBITDA $2.97B, net loss $407M on a $556M non-cash India regulatory impairment</t>
+        </is>
+      </c>
+      <c r="CY4" t="n">
+        <v>4</v>
+      </c>
+      <c r="CZ4" t="n">
+        <v>4</v>
+      </c>
+      <c r="DA4" t="n">
+        <v>5</v>
+      </c>
+      <c r="DB4" t="n">
+        <v>2</v>
+      </c>
+      <c r="DC4" t="n">
+        <v>5</v>
+      </c>
+      <c r="DD4" t="n">
+        <v>80</v>
+      </c>
+      <c r="DE4" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="DH4" t="inlineStr">
+        <is>
+          <t>https://www.globenewswire.com/news-release/2026/02/26/3246102/0/en/flutter-entertainment-reports-fourth-quarter-and-full-year-2025-financial-results.html ; https://infotechlead.com/gaming/flutter-accelerates-ai-driven-betting-tech-and-fanduel-one-app-strategy-in-2026-95681 ; https://flutter.com/news-media/blogs/huddle-up-recap-inside-fanduel-s-50-billion-playbook/ ; https://www.covers.com/industry/fanduel-again-tops-sportsbook-q2-earnings-august-11-2025</t>
+        </is>
+      </c>
+      <c r="DI4" t="inlineStr">
+        <is>
+          <t>Strong recent disclosure via SEC 8-K/earnings releases and multiple corroborating trade press; AI-specific claims (foundation model depth, agentic maturity) inferred from limited product detail. || W1=4: FanDuel Predicts/One App repositions strategy around owned demand | W2=4: ≈$300M FanDuel Predicts investment plus CME JV, One App build | W3=4: CME Group JV reaches 40% of underserved US population | W4=5: FanDuel One App live Apr 2026: unified sportsbook+predictions+casino surface | W5=5: 15.9M monthly players; 43% US sportsbook share, dominant app reach | D1=5: Sportsbook, casino, poker (PokerStars), lottery across multiple leading brands | D2=5: Proprietary pricing/risk tech now commercialized to third-party prediction venues | D3=5: Multi-jurisdiction: US states, UK, Ireland, Italy, Australia, Brazil, India | D4=3: Payments infra not publicly confirmed as owned MoR at scale | D5=5: $18.4B FY25 revenue, global multi-brand footprint, millions of actives | D6=5: FanDuel #1 US brand; Paddy Power/Betfair trusted UK heritage brands | AI1=3: Proprietary pricing/risk models sold to third parties; no confirmed frontier LLMs | AI2=1: No shipped autonomous betting agent found; personalization tools only | AI3=0: No MCP/A2A/UCP/ACP adoption evidence found | AI4=2: Bet Protect+ AI promo tool shipped; no full chat assistant | AI5=4: Bet Protect+ adoption 2x forecast; predictive analytics across brands | AI6=5: 15.9M actives, multi-vertical global data now sold as B2B service | AI7=3: Sells pricing/risk tech to CME-linked prediction venues as provider | F1=4: Adj EBITDA $2.97B FY25, strong operating cash generation, well-funded | F2=4: $18.4B revenue +19%, but $407M net loss from India impairment | F3=5: Scaled, cash-generative multinational operator; no near-term funding risk | F4=2: Comparison source cites Flutter's ~$10.6bn net debt as leveraged | F5=5: NYSE/LSE dual-listed large-cap; proven access to capital markets</t>
+        </is>
+      </c>
+      <c r="DJ4" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="DK4" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="DL4" t="inlineStr">
+        <is>
+          <t>sonnet/company-researcher</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Betsson AB (publ)</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Stockholm, Sweden (group operations via Malta)</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1963</v>
+      </c>
+      <c r="F5" t="n">
+        <v>2160</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Operator (B2C)</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Multi-brand online sportsbook/casino operator (Betsafe, Betsson.com, Rizk, NordicBet and others) monetizing GGR, with a growing share of revenue from newly locally-regulated markets, plus a smaller B2B platform business.</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>B2C — sports bettors and casino players, strongest in Nordics, Latin America (Brazil, Paraguay, Argentina) and other European markets</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>External vendor AI (Ada) for customer-service chat; no evidence of own model development</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>600k+ active customers across 24 licensed markets; standard transactional/CRM data, no described data moat</t>
+        </is>
+      </c>
+      <c r="AF5" t="inlineStr">
+        <is>
+          <t>Ada (AI chatbot platform vendor)</t>
+        </is>
+      </c>
+      <c r="AH5" t="inlineStr">
+        <is>
+          <t>24 licensed markets including Sweden and other Nordics, Brazil, Paraguay, Argentina, and various EU jurisdictions</t>
+        </is>
+      </c>
+      <c r="AI5" t="n">
+        <v>68</v>
+      </c>
+      <c r="AK5" t="inlineStr">
+        <is>
+          <t>Standard safer-gambling tools tied to licence conditions across its 24 regulated markets; not independently verified this session</t>
+        </is>
+      </c>
+      <c r="AM5" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AN5" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AO5" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AP5" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AQ5" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AR5" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AS5" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AT5" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AV5" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AZ5" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="BB5" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="BD5" t="n">
+        <v>3</v>
+      </c>
+      <c r="BI5" t="n">
+        <v>1</v>
+      </c>
+      <c r="BJ5" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK5" t="n">
+        <v>1</v>
+      </c>
+      <c r="BL5" t="n">
+        <v>1</v>
+      </c>
+      <c r="BM5" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN5" t="n">
+        <v>3</v>
+      </c>
+      <c r="BO5" t="n">
+        <v>4</v>
+      </c>
+      <c r="BP5" t="n">
+        <v>4</v>
+      </c>
+      <c r="BQ5" t="n">
+        <v>3</v>
+      </c>
+      <c r="BR5" t="n">
+        <v>4</v>
+      </c>
+      <c r="BS5" t="n">
+        <v>3</v>
+      </c>
+      <c r="BT5" t="n">
+        <v>2</v>
+      </c>
+      <c r="BU5" t="n">
+        <v>1</v>
+      </c>
+      <c r="BV5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW5" t="n">
+        <v>3</v>
+      </c>
+      <c r="BX5" t="n">
+        <v>2</v>
+      </c>
+      <c r="BY5" t="n">
+        <v>2</v>
+      </c>
+      <c r="BZ5" t="n">
+        <v>1</v>
+      </c>
+      <c r="CA5" t="n">
+        <v>20</v>
+      </c>
+      <c r="CB5" t="n">
+        <v>70</v>
+      </c>
+      <c r="CC5" t="n">
+        <v>30</v>
+      </c>
+      <c r="CD5" t="n">
+        <v>50</v>
+      </c>
+      <c r="CE5" t="n">
+        <v>38</v>
+      </c>
+      <c r="CF5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="CG5" t="inlineStr">
+        <is>
+          <t>Dormant</t>
+        </is>
+      </c>
+      <c r="CH5" t="inlineStr">
+        <is>
+          <t>No owned acquisition surface or agentic AI; relies on affiliate/brand marketing and a vendor chatbot only.</t>
+        </is>
+      </c>
+      <c r="CJ5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="CK5" t="inlineStr">
+        <is>
+          <t>3y+</t>
+        </is>
+      </c>
+      <c r="CL5" t="inlineStr">
+        <is>
+          <t>Betsson exemplifies the incumbent archetype itself — defensive, distribution-strong, using AI for CRM/efficiency rather than player-ownership.</t>
+        </is>
+      </c>
+      <c r="CN5" t="inlineStr">
+        <is>
+          <t>Legal entity Betsson AB (publ), Nasdaq Stockholm (BETS B); founded 1963 as AB Restaurang Rouletter, renamed Betsson 2001. Marked in the project seedlist as the sector's 'reference competitor set' anchor — used here as the incumbent-archetype baseline rather than a disruption-forward company.</t>
+        </is>
+      </c>
+      <c r="CQ5" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="CU5" t="inlineStr">
+        <is>
+          <t>Record €1.197B FY2025 revenue (+8% YoY), EBITDA €313.7M (margin 26.2%, down from 28.6%), net income €182.4M</t>
+        </is>
+      </c>
+      <c r="CY5" t="n">
+        <v>4</v>
+      </c>
+      <c r="CZ5" t="n">
+        <v>4</v>
+      </c>
+      <c r="DA5" t="n">
+        <v>5</v>
+      </c>
+      <c r="DB5" t="n">
+        <v>3</v>
+      </c>
+      <c r="DC5" t="n">
+        <v>4</v>
+      </c>
+      <c r="DD5" t="n">
+        <v>80</v>
+      </c>
+      <c r="DE5" t="inlineStr">
+        <is>
+          <t>Stable</t>
+        </is>
+      </c>
+      <c r="DH5" t="inlineStr">
+        <is>
+          <t>https://gamblersconnect.com/news/finance/betsson-2025-annual-report/ ; https://next.io/news/technology/betsson-fredrik-ogren-cleber-de-lima-interview-ai-adoption/ ; https://www.digitaljournal.com/article/betsson-drives-customer-service-with-ada-ai-powered-chatbots/ ; https://www.betssonab.com/about-us/strategy</t>
+        </is>
+      </c>
+      <c r="DI5" t="inlineStr">
+        <is>
+          <t>Financials well-documented via annual/year-end report; willingness and AI-depth signals rely on thinner trade-press coverage (chatbot vendor deployment, CTO interview) — likely understates any undisclosed internal AI work. || W1=1: Content with current model; AI framed as efficiency, not acquisition disruption | W2=1: M&amp;A (Rhino Canada, Sporting Solutions) targets scale, not AI/wallet disruption | W3=1: Ada is a vendor relationship, not a distribution alliance | W4=1: Only shipped experiment: Ada AI customer-service chatbot across brands | W5=1: 600k+ actives acquired via conventional brand/affiliate marketing, not owned intent | D1=3: Multi-brand sportsbook/casino; content largely licensed-in from B2B suppliers | D2=4: Own proprietary tech platform cited as top strategic priority | D3=4: 24 licensed markets; 68% of revenue now locally regulated | D4=3: Payments via partner rails; no confirmed owned MoR status | D5=4: €1.197B revenue, LatAm+Nordics+EU footprint, record local-licence share | D6=3: Respected mid-tier brand in core markets, not globally top-of-mind | AI1=2: Uses third-party AI platform (Ada) for chatbots; no own models found | AI2=1: Self-serve chatbot only; no autonomous transaction capability shown | AI3=0: No agent-commerce protocol adoption evidence found | AI4=3: Ada chatbots serve 600k+ actives in 8 languages, 24/7 | AI5=2: Predictive tools for CRM/bonusing mentioned; no individual-level detail found | AI6=2: Standard transactional/CRM data; no described proprietary data moat | AI7=1: Pure consumer of vendor AI (Ada); no platform position | F1=4: EBITDA €313.7M FY25; profitable, no funding gap evident | F2=4: Record €1.197B revenue +8%; EBITDA margin dipped to 26.2% | F3=5: Consistently profitable, self-funding operator; no runway concern | F4=3: No explicit leverage data found; small M&amp;A self-funded in cash | F5=4: Nasdaq Stockholm listed; established public capital-market access</t>
+        </is>
+      </c>
+      <c r="DJ5" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="DK5" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="DL5" t="inlineStr">
+        <is>
+          <t>sonnet/company-researcher</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Bet365 Group Ltd</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Stoke-on-Trent, UK</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F6" t="n">
+        <v>12000</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Operator (B2C)</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Private, family-owned global sportsbook/casino operator trading as Hillside (New Media) Limited, self-funded from internal cash flow, monetizing GGR with no external investors or debt.</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>B2C — global sports bettors and casino players; legal in 80+ countries, directly licensed in 30+</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>In-house ML for a new AI-driven betting platform ($50M investment, launching 2026); no evidence of frontier model training</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>Decades of proprietary in-house odds-setting and in-play pricing data at global scale; exact scope undisclosed (private company)</t>
+        </is>
+      </c>
+      <c r="AF6" t="inlineStr">
+        <is>
+          <t>TestMu AI (agentic QA/test engineering vendor)</t>
+        </is>
+      </c>
+      <c r="AH6" t="inlineStr">
+        <is>
+          <t>UK Gambling Commission, Malta Gaming Authority plus 30+ direct licences; legally available in 80+ countries; live in 16 US states</t>
+        </is>
+      </c>
+      <c r="AK6" t="inlineStr">
+        <is>
+          <t>Uses AI-driven systems to flag problem-gambling patterns and trigger deposit-limit/self-exclusion prompts</t>
+        </is>
+      </c>
+      <c r="AM6" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AN6" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AO6" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AP6" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AQ6" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AR6" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AS6" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AT6" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AV6" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AZ6" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="BB6" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="BD6" t="n">
+        <v>4</v>
+      </c>
+      <c r="BI6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BJ6" t="n">
+        <v>2</v>
+      </c>
+      <c r="BK6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BL6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BM6" t="n">
+        <v>2</v>
+      </c>
+      <c r="BN6" t="n">
+        <v>5</v>
+      </c>
+      <c r="BO6" t="n">
+        <v>5</v>
+      </c>
+      <c r="BP6" t="n">
+        <v>5</v>
+      </c>
+      <c r="BQ6" t="n">
+        <v>3</v>
+      </c>
+      <c r="BR6" t="n">
+        <v>5</v>
+      </c>
+      <c r="BS6" t="n">
+        <v>5</v>
+      </c>
+      <c r="BT6" t="n">
+        <v>2</v>
+      </c>
+      <c r="BU6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BV6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX6" t="n">
+        <v>2</v>
+      </c>
+      <c r="BY6" t="n">
+        <v>4</v>
+      </c>
+      <c r="BZ6" t="n">
+        <v>1</v>
+      </c>
+      <c r="CA6" t="n">
+        <v>27</v>
+      </c>
+      <c r="CB6" t="n">
+        <v>94</v>
+      </c>
+      <c r="CC6" t="n">
+        <v>30</v>
+      </c>
+      <c r="CD6" t="n">
+        <v>62</v>
+      </c>
+      <c r="CE6" t="n">
+        <v>48</v>
+      </c>
+      <c r="CF6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="CG6" t="inlineStr">
+        <is>
+          <t>Sleeping giant</t>
+        </is>
+      </c>
+      <c r="CH6" t="inlineStr">
+        <is>
+          <t>No shipped conversational/agentic AI product; extreme corporate opacity limits verification of willingness and AI claims.</t>
+        </is>
+      </c>
+      <c r="CJ6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="CK6" t="inlineStr">
+        <is>
+          <t>1-3y</t>
+        </is>
+      </c>
+      <c r="CL6" t="inlineStr">
+        <is>
+          <t>Bet365 is the most distribution-dominant incumbent in the set, but its low willingness to disrupt its own model keeps it a 'sleeping giant' relative to Flutter/DraftKings.</t>
+        </is>
+      </c>
+      <c r="CN6" t="inlineStr">
+        <is>
+          <t>Legal entity Bet365 Group Ltd; UK operations trade as Hillside (New Media) Limited within the umbrella 'Hillside Group'. Wholly private, Coates family owned (Denise Coates ~58%, John Coates ~25%, Peter Coates chairman/remainder). No ticker, no public market cap — market_cap_valuation_mn is a third-party private valuation estimate (Eilers &amp; Krejcik midpoint, ~2025), not a listed figure. Confidence capped at medium given reliance on UK filings/press rather than company disclosure.</t>
+        </is>
+      </c>
+      <c r="CQ6" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="CU6" t="inlineStr">
+        <is>
+          <t>£4.036B group revenue for FY ended 30 March 2025 (+9% YoY); pre-tax profit fell 44% to £348.7M</t>
+        </is>
+      </c>
+      <c r="CY6" t="n">
+        <v>5</v>
+      </c>
+      <c r="CZ6" t="n">
+        <v>3</v>
+      </c>
+      <c r="DA6" t="n">
+        <v>5</v>
+      </c>
+      <c r="DB6" t="n">
+        <v>5</v>
+      </c>
+      <c r="DC6" t="n">
+        <v>3</v>
+      </c>
+      <c r="DD6" t="n">
+        <v>84</v>
+      </c>
+      <c r="DE6" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="DH6" t="inlineStr">
+        <is>
+          <t>https://wageringamerica.com/2026/06/07/bet365-equity-research-jun-2026/ ; https://sbcamericas.com/2025/05/01/coates-considers-sale-spinoff-bet365/ ; https://www.bestinslot.co/news/bet365-announces-groundbreaking-50-million-investment-in-ai-driven-betting-platform-19839 ; https://www.businesswire.com/news/home/20260331630451/en/bet365-Partners-with-TestMu-AI-to-Accelerate-Global-Release-Velocity-with-Agentic-AI-Quality-Engineering</t>
+        </is>
+      </c>
+      <c r="DI6" t="inlineStr">
+        <is>
+          <t>Good visibility on financials via UK Companies House-derived press coverage and equity-research notes; strategy and AI-depth claims rely on sparse press releases since the company does not hold investor calls or publish detailed disclosures. || W1=1: Focused on improving existing sportsbook, not attacking acquisition model | W2=2: $50M investment in new AI-driven betting platform, launching early 2026 | W3=1: TestMu AI is engineering/QA tooling, not a distribution alliance | W4=1: New AI platform not yet fully live as of mid-2026 | W5=2: Reputedly low affiliate spend/strong organic reach; no public MAU data | D1=5: Industry-leading in-play betting breadth across sports, casino, poker, bingo | D2=5: Hillside Technology's own platform ships hundreds of releases weekly | D3=5: Licensed 30+ jurisdictions directly; legally live in 80+ countries | D4=3: Handles payments across many markets; MoR structure not disclosed | D5=5: £4.036B revenue, global 80+ country reach, 16 US states | D6=5: Globally recognized, trusted brand; leader in odds-setting reputation | AI1=2: ML-driven platform under $50M investment; no frontier model evidence | AI2=1: AI platform pre-launch/early rollout; no shown autonomy yet | AI3=0: No MCP/A2A/UCP/ACP adoption evidence found | AI4=0: No confirmed customer-facing conversational assistant product identified | AI5=2: New platform targets personalized odds/UX; still rolling out in 2026 | AI6=4: Decades of proprietary in-house pricing/trading data at global scale | AI7=1: TestMu partnership is vendor consumption, not an AI platform position | F1=5: Self-funded from ~£3.1bn cash; no external financing needed | F2=3: Revenue +9% to £4.036B but pre-tax profit fell 44% | F3=5: Zero debt, £3.1bn liquidity; effectively unlimited runway | F4=5: Debt-free since 2005; no external leverage per multiple sources | F5=3: Private; no public markets, though PE sale/listing explored in 2025</t>
+        </is>
+      </c>
+      <c r="DJ6" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="DK6" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="DL6" t="inlineStr">
+        <is>
+          <t>sonnet/company-researcher</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Entain plc</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>London, UK (registered office Isle of Man)</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>2004</v>
+      </c>
+      <c r="F7" t="n">
+        <v>6400</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Operator (B2C)</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Multi-brand sportsbook/casino operator (Ladbrokes, Coral, bwin, partypoker, Sportingbet) monetizing GGR; BetMGM is a 50/50 US joint venture with MGM Resorts International.</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>B2C — sports bettors and casino players across UK/Ireland and 30+ international regulated markets, plus US via the BetMGM joint venture</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>External platform AI (Snowflake Cortex) for internal software-delivery tooling; no evidence of own model training</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>L0</t>
+        </is>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>Behavioral/transaction data across 30+ regulated markets plus BetMGM US JV; no described unique data moat found</t>
+        </is>
+      </c>
+      <c r="AF7" t="inlineStr">
+        <is>
+          <t>MGM Resorts International (BetMGM 50/50 JV), Snowflake, LTIMindtree</t>
+        </is>
+      </c>
+      <c r="AH7" t="inlineStr">
+        <is>
+          <t>UK, Ireland, Italy, Belgium, Netherlands, Croatia, Poland, Georgia, Latvia, Australia (wholly owned) plus US via BetMGM JV; 30+ regulated markets total</t>
+        </is>
+      </c>
+      <c r="AI7" t="n">
+        <v>100</v>
+      </c>
+      <c r="AK7" t="inlineStr">
+        <is>
+          <t>States it operates exclusively in domestically regulated/regulating markets; standard safer-gambling tooling implied, not independently detailed this session</t>
+        </is>
+      </c>
+      <c r="AM7" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AN7" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AO7" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AP7" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AQ7" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AR7" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AS7" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AT7" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AV7" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AX7" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AZ7" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="BB7" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="BD7" t="n">
+        <v>4</v>
+      </c>
+      <c r="BI7" t="n">
+        <v>1</v>
+      </c>
+      <c r="BJ7" t="n">
+        <v>3</v>
+      </c>
+      <c r="BK7" t="n">
+        <v>1</v>
+      </c>
+      <c r="BL7" t="n">
+        <v>1</v>
+      </c>
+      <c r="BM7" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN7" t="n">
+        <v>4</v>
+      </c>
+      <c r="BO7" t="n">
+        <v>4</v>
+      </c>
+      <c r="BP7" t="n">
+        <v>5</v>
+      </c>
+      <c r="BQ7" t="n">
+        <v>3</v>
+      </c>
+      <c r="BR7" t="n">
+        <v>4</v>
+      </c>
+      <c r="BS7" t="n">
+        <v>4</v>
+      </c>
+      <c r="BT7" t="n">
+        <v>2</v>
+      </c>
+      <c r="BU7" t="n">
+        <v>1</v>
+      </c>
+      <c r="BV7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX7" t="n">
+        <v>2</v>
+      </c>
+      <c r="BY7" t="n">
+        <v>2</v>
+      </c>
+      <c r="BZ7" t="n">
+        <v>1</v>
+      </c>
+      <c r="CA7" t="n">
+        <v>30</v>
+      </c>
+      <c r="CB7" t="n">
+        <v>80</v>
+      </c>
+      <c r="CC7" t="n">
+        <v>24</v>
+      </c>
+      <c r="CD7" t="n">
+        <v>52</v>
+      </c>
+      <c r="CE7" t="n">
+        <v>43</v>
+      </c>
+      <c r="CF7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="CG7" t="inlineStr">
+        <is>
+          <t>Dormant</t>
+        </is>
+      </c>
+      <c r="CH7" t="inlineStr">
+        <is>
+          <t>No owned AI-native acquisition surface; leverage and a UK tax-driven impairment constrain capital for offensive bets.</t>
+        </is>
+      </c>
+      <c r="CJ7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="CK7" t="inlineStr">
+        <is>
+          <t>3y+</t>
+        </is>
+      </c>
+      <c r="CL7" t="inlineStr">
+        <is>
+          <t>Entain is squarely the incumbent under pressure — BetMGM's repeated guidance cuts show prediction markets eroding its position rather than Entain leading disruption.</t>
+        </is>
+      </c>
+      <c r="CN7" t="inlineStr">
+        <is>
+          <t>Legal entity Entain plc (LSE: ENT), founded 2004 as Gaming VC Holdings (GVC Holdings), renamed Entain in December 2020. BetMGM LLC is a 50/50 joint venture with MGM Resorts International — scored at the Entain parent level; BetMGM performance included for context only, not counted as wholly-owned distribution or willingness.</t>
+        </is>
+      </c>
+      <c r="CQ7" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="CU7" t="inlineStr">
+        <is>
+          <t>£5,325.4m NGR FY2025 (+3-4% YoY), underlying EBITDA £1,160.1m (+7-8%), net loss £680.5m including a £488m UK gambling-tax-related impairment</t>
+        </is>
+      </c>
+      <c r="CY7" t="n">
+        <v>3</v>
+      </c>
+      <c r="CZ7" t="n">
+        <v>2</v>
+      </c>
+      <c r="DA7" t="n">
+        <v>3</v>
+      </c>
+      <c r="DB7" t="n">
+        <v>2</v>
+      </c>
+      <c r="DC7" t="n">
+        <v>4</v>
+      </c>
+      <c r="DD7" t="n">
+        <v>56</v>
+      </c>
+      <c r="DE7" t="inlineStr">
+        <is>
+          <t>Stable</t>
+        </is>
+      </c>
+      <c r="DH7" t="inlineStr">
+        <is>
+          <t>https://www.entaingroup.com/news-insights/latest-news/2026/2025-full-year-results/ ; https://www.gamblinginsider.com/news/179065/betmgm-q2-2026-earnings-prediction-markets-customer-win-rates-weigh-on-results ; https://sbcnews.co.uk/technology/2025/07/08/entain-india-tech-arm/ ; https://ggbmagazine.com/articles/entain-launches-innovation-hub/</t>
+        </is>
+      </c>
+      <c r="DI7" t="inlineStr">
+        <is>
+          <t>Official FY2025 results release gives solid financial grounding; AI-specific and willingness signals rely on secondary trade press (tech-hub, Snowflake blog) and inference from BetMGM's defensive posture against prediction markets. || W1=1: Reactive to prediction-market pressure on BetMGM, not proactively offensive | W2=3: Ennovate hub commits up to £100M to innovation/startup investment | W3=1: Partnerships (Snowflake, LTIMindtree) are infra vendors, not distribution deals | W4=1: No flagship owned AI/wallet/prediction surface identified beyond standard apps | W5=1: Acquisition remains brand/affiliate-driven across Ladbrokes, Coral, bwin, BetMGM | D1=4: Sportsbook, casino, poker, bingo across Ladbrokes/Coral/bwin/partypoker/BetMGM brands | D2=4: Long-invested unified platform infrastructure across international brand portfolio | D3=5: 30+ regulated markets; 100% of revenue from regulated/regulating markets | D4=3: Payments via partner networks typical of sector; MoR status unconfirmed | D5=4: £5.3B revenue, top-3 position in 87%+ of revenue markets | D6=4: Ladbrokes/Coral are trusted UK high-street heritage betting brands | AI1=2: Uses Snowflake Cortex GenAI for SDLC; API/platform consumer tier | AI2=1: No customer-facing autonomous agent found; internal tooling only | AI3=0: No agent-commerce protocol adoption evidence found | AI4=0: No confirmed customer-facing conversational assistant identified | AI5=2: Pune hub cited for AI-driven personalisation; segment-level, unconfirmed depth | AI6=2: Large multi-market dataset incl. BetMGM US; no described unique moat | AI7=1: Consumer of Snowflake/LTIMindtree AI tools, not an AI platform provider | F1=3: Underlying EBITDA £1.16B positive, but reported £680.5M net loss | F2=2: Revenue/EBITDA grew modestly, but net loss on UK tax impairment | F3=3: Ongoing EBITDA-positive operations, but high leverage adds fragility | F4=2: Net debt £3,644m; leverage 3.1x, look-through 3.6x | F5=4: LSE-listed large-cap; established access to public capital markets</t>
+        </is>
+      </c>
+      <c r="DJ7" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="DK7" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="DL7" t="inlineStr">
+        <is>
+          <t>sonnet/company-researcher</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>DraftKings Inc.</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Boston, Massachusetts, US</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>2012</v>
+      </c>
+      <c r="F8" t="n">
+        <v>12360</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Operator (B2C)</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>US-focused sportsbook/casino/lottery operator (plus legacy DFS) monetizing GGR; expanding into CFTC-licensed prediction markets through the Railbird acquisition and DraftKings Predictions, moving toward a unified 'Super App'.</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>B2C — US sports bettors, casino/DFS players and lottery customers; essentially a single-country (US) consumer base</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>External AI tools/APIs for coding, RFPs, ops and chat; no evidence of own model training</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t>Legacy DFS entry/contest data plus the widest US state-sportsbook footprint; no industry-defining moat described</t>
+        </is>
+      </c>
+      <c r="AF8" t="inlineStr">
+        <is>
+          <t>CME Group, Crypto.com (prediction-market contracts), Railbird (acquired Oct 2025), MaestroQA (AI coaching vendor)</t>
+        </is>
+      </c>
+      <c r="AH8" t="inlineStr">
+        <is>
+          <t>27 US states plus Washington DC for online sportsbook (widest state coverage of any US operator); lottery via Jackpocket in additional states</t>
+        </is>
+      </c>
+      <c r="AK8" t="inlineStr">
+        <is>
+          <t>Standard US state-licence safer-gambling requirements; not independently detailed this session</t>
+        </is>
+      </c>
+      <c r="AL8" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AM8" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AN8" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AO8" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AP8" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AQ8" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AR8" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AS8" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AT8" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AV8" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AX8" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AZ8" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="BB8" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="BD8" t="n">
+        <v>4</v>
+      </c>
+      <c r="BI8" t="n">
+        <v>4</v>
+      </c>
+      <c r="BJ8" t="n">
+        <v>4</v>
+      </c>
+      <c r="BK8" t="n">
+        <v>3</v>
+      </c>
+      <c r="BL8" t="n">
+        <v>4</v>
+      </c>
+      <c r="BM8" t="n">
+        <v>4</v>
+      </c>
+      <c r="BN8" t="n">
+        <v>4</v>
+      </c>
+      <c r="BO8" t="n">
+        <v>4</v>
+      </c>
+      <c r="BP8" t="n">
+        <v>3</v>
+      </c>
+      <c r="BQ8" t="n">
+        <v>3</v>
+      </c>
+      <c r="BR8" t="n">
+        <v>2</v>
+      </c>
+      <c r="BS8" t="n">
+        <v>4</v>
+      </c>
+      <c r="BT8" t="n">
+        <v>2</v>
+      </c>
+      <c r="BU8" t="n">
+        <v>1</v>
+      </c>
+      <c r="BV8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW8" t="n">
+        <v>2</v>
+      </c>
+      <c r="BX8" t="n">
+        <v>2</v>
+      </c>
+      <c r="BY8" t="n">
+        <v>3</v>
+      </c>
+      <c r="BZ8" t="n">
+        <v>1</v>
+      </c>
+      <c r="CA8" t="n">
+        <v>76</v>
+      </c>
+      <c r="CB8" t="n">
+        <v>70</v>
+      </c>
+      <c r="CC8" t="n">
+        <v>31</v>
+      </c>
+      <c r="CD8" t="n">
+        <v>50</v>
+      </c>
+      <c r="CE8" t="n">
+        <v>60</v>
+      </c>
+      <c r="CF8" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="CG8" t="inlineStr">
+        <is>
+          <t>Aspirant</t>
+        </is>
+      </c>
+      <c r="CH8" t="inlineStr">
+        <is>
+          <t>No international scale or licensing; the DraftKings Exchange and full Super App integration are still mid-rollout, not fully proven.</t>
+        </is>
+      </c>
+      <c r="CJ8" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="CK8" t="inlineStr">
+        <is>
+          <t>0-12m</t>
+        </is>
+      </c>
+      <c r="CL8" t="inlineStr">
+        <is>
+          <t>DraftKings is racing alongside Flutter/FanDuel to own the prediction-markets flank before it cannibalizes traditional sportsbook margin from outside the licensing regime.</t>
+        </is>
+      </c>
+      <c r="CN8" t="inlineStr">
+        <is>
+          <t>Legal entity DraftKings Inc (NASDAQ: DKNG). Acquired Jackpocket (lottery courier, 2024) and Railbird Technologies/Railbird Exchange (CFTC-licensed prediction platform, closed Oct 2025) — both now subsidiaries, not separate entities. Essentially a US-only operator, unlike the other four multinational operators in this batch — flag when comparing D5 global-scale and W5 audience-scale scores across the set.</t>
+        </is>
+      </c>
+      <c r="CQ8" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="CU8" t="inlineStr">
+        <is>
+          <t>$6.05B FY2025 revenue (+27% YoY), adjusted EBITDA $620M (+242.5% YoY), first positive net income since its 2020 IPO</t>
+        </is>
+      </c>
+      <c r="CY8" t="n">
+        <v>4</v>
+      </c>
+      <c r="CZ8" t="n">
+        <v>4</v>
+      </c>
+      <c r="DA8" t="n">
+        <v>4</v>
+      </c>
+      <c r="DC8" t="n">
+        <v>4</v>
+      </c>
+      <c r="DD8" t="n">
+        <v>80</v>
+      </c>
+      <c r="DE8" t="inlineStr">
+        <is>
+          <t>Stable</t>
+        </is>
+      </c>
+      <c r="DH8" t="inlineStr">
+        <is>
+          <t>https://next.io/news/prediction-markets/draftkings-seals-railbird-acquisition-prediction-markets-launch/ ; https://www.cnbc.com/2025/10/21/draftkings-railbird-predictions-platform-acquisition.html ; https://www.covers.com/industry/draftkings-to-offer-users-crypto-to-cash-access-in-4-states-feb-2-2026 ; https://www.covers.com/industry/draftkings-finishes-2025-on-high-note-increases-q4-revenue-feb-12-2026</t>
+        </is>
+      </c>
+      <c r="DI8" t="inlineStr">
+        <is>
+          <t>Strong recent disclosure via earnings coverage and multiple corroborating trade-press sources on Railbird/prediction-markets strategy; AI-depth and leverage/debt-structure claims are thinner and partly inferred. || W1=4: Building 'Super App' unifying sportsbook, casino, lottery, predictions as core strategy | W2=4: Acquired Railbird (CFTC-licensed exchange); investing to reduce third-party dependence | W3=3: CME/Crypto.com contract deals, though moving toward owned-exchange independence | W4=4: DraftKings Predictions live Dec 2025; crypto-to-cash deposits in 4 states | W5=4: Widest US state footprint (27+DC); #2 US sportsbook operator by scale | D1=4: Sportsbook, casino, lottery (Jackpocket), now prediction markets via Railbird | D2=4: Owns Railbird exchange tech; platform historically built via SBTech acquisition | D3=3: 27 states + DC; strong domestic breadth, no international scale | D4=3: Crypto-to-cash deposits in 4 states; fiat MoR status unclear | D5=2: $6.05B revenue but essentially US-only; no material global footprint | D6=4: #2 US betting brand by revenue/EBITDA behind FanDuel, well recognized | AI1=2: AI used for coding, RFPs, ops efficiency via external tools, not own models | AI2=1: AI-powered coaching (MaestroQA) and chatbots are assistive, not autonomous | AI3=0: No MCP/A2A/UCP/ACP adoption evidence found | AI4=2: Chatbots implemented for customer service per trade-press coverage | AI5=2: AI cited for personalized content serving; depth/scope not detailed | AI6=3: Legacy DFS entry data plus widest-state sportsbook behavioral dataset | AI7=1: Consumer of AI vendors (MaestroQA, coding tools), not an AI platform provider | F1=4: Adj EBITDA $620M FY25, up 242.5%; funding position much improved | F2=4: Revenue $6.05B +27%; first-ever positive net income since 2020 IPO | F3=4: Newly cash-generative and profitable; runway concerns much reduced | F4=None: Leverage/debt structure not confirmed via sources found this session | F5=4: NASDAQ large-cap ($12.36B mkt cap); proven equity/convert capital access</t>
+        </is>
+      </c>
+      <c r="DJ8" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="DK8" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="DL8" t="inlineStr">
+        <is>
+          <t>sonnet/company-researcher</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Evolution AB (publ)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Stockholm, Sweden</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>2006</v>
+      </c>
+      <c r="D9" t="n">
+        <v>16243</v>
+      </c>
+      <c r="F9" t="n">
+        <v>13400</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>B2B supplier &amp; platform</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>B2B live-casino and RNG-slot content licensor to 800+ operators worldwide; earns royalty/commission on operator handle, not player-facing.</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>B2B — licensed gambling operators worldwide (not B2C)</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t>L0</t>
+        </is>
+      </c>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>Cross-operator live-dealer behavioral/session data at massive scale</t>
+        </is>
+      </c>
+      <c r="AF9" t="inlineStr">
+        <is>
+          <t>NetEnt, Red Tiger, Ezugi, Big Time Gaming, DigiWheel (subsidiaries); 800+ licensed operators as customers</t>
+        </is>
+      </c>
+      <c r="AH9" t="inlineStr">
+        <is>
+          <t>Supplier-licensed across most regulated tier-1 markets; UK licence under active UKGC review (2025)</t>
+        </is>
+      </c>
+      <c r="AK9" t="inlineStr">
+        <is>
+          <t>Standard supplier-level RG tooling; UKGC currently reviewing licence over unlicensed-market access allegations</t>
+        </is>
+      </c>
+      <c r="AM9" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AN9" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AO9" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AP9" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AQ9" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AR9" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AS9" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AT9" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AV9" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AX9" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AZ9" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="BB9" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="BD9" t="n">
+        <v>2</v>
+      </c>
+      <c r="BI9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ9" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK9" t="n">
+        <v>1</v>
+      </c>
+      <c r="BL9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN9" t="n">
+        <v>5</v>
+      </c>
+      <c r="BO9" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP9" t="n">
+        <v>4</v>
+      </c>
+      <c r="BQ9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BR9" t="n">
+        <v>5</v>
+      </c>
+      <c r="BS9" t="n">
+        <v>3</v>
+      </c>
+      <c r="BT9" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX9" t="n">
+        <v>1</v>
+      </c>
+      <c r="BY9" t="n">
+        <v>3</v>
+      </c>
+      <c r="BZ9" t="n">
+        <v>1</v>
+      </c>
+      <c r="CA9" t="n">
+        <v>9</v>
+      </c>
+      <c r="CB9" t="n">
+        <v>58</v>
+      </c>
+      <c r="CC9" t="n">
+        <v>16</v>
+      </c>
+      <c r="CD9" t="n">
+        <v>37</v>
+      </c>
+      <c r="CE9" t="n">
+        <v>26</v>
+      </c>
+      <c r="CF9" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="CG9" t="inlineStr">
+        <is>
+          <t>Dormant</t>
+        </is>
+      </c>
+      <c r="CH9" t="inlineStr">
+        <is>
+          <t>No player-facing wallet, brand, or acquisition channel — deliberately stays B2B-only</t>
+        </is>
+      </c>
+      <c r="CJ9" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="CK9" t="inlineStr">
+        <is>
+          <t>3y+</t>
+        </is>
+      </c>
+      <c r="CL9" t="inlineStr">
+        <is>
+          <t>Indispensable content rail incumbents depend on; zero ambition to own the player relationship</t>
+        </is>
+      </c>
+      <c r="CN9" t="inlineStr">
+        <is>
+          <t>Legal entity Evolution AB (publ), Nasdaq Stockholm ticker EVO. Subsidiaries NetEnt, Red Tiger, Ezugi, Big Time Gaming, DigiWheel are consolidated under this parent — not separate rows. UKGC licence review (2025) over allegations its games appeared on unlicensed UK-facing sites is a live compliance flag, not yet resolved.</t>
+        </is>
+      </c>
+      <c r="CQ9" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="CU9" t="inlineStr">
+        <is>
+          <t>FY2025 revenue record &gt;EUR2.4bn; Q1 2026 revenue ~EUR538M, +16% YoY</t>
+        </is>
+      </c>
+      <c r="CY9" t="n">
+        <v>5</v>
+      </c>
+      <c r="CZ9" t="n">
+        <v>5</v>
+      </c>
+      <c r="DA9" t="n">
+        <v>5</v>
+      </c>
+      <c r="DB9" t="n">
+        <v>4</v>
+      </c>
+      <c r="DC9" t="n">
+        <v>5</v>
+      </c>
+      <c r="DD9" t="n">
+        <v>96</v>
+      </c>
+      <c r="DE9" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="DH9" t="inlineStr">
+        <is>
+          <t>https://www.ad-hoc-news.de/boerse/news/ueberblick/evolution-stock-trades-around-yearly-highs-as-strong-q1-2026-earnings/69819209 ; https://stockanalysis.com/quote/sto/EVO/market-cap/ ; https://next.io/news/regulation/ukgc-commences-review-evolution-licence/ ; https://en.wikipedia.org/wiki/Evolution_AB</t>
+        </is>
+      </c>
+      <c r="DI9" t="inlineStr">
+        <is>
+          <t>Evidence from Q1/Q2 2026 earnings coverage, market-cap trackers, and UKGC review reporting. Direct fetch of Evolution's own IR site failed (blocked); relied on secondary aggregator coverage of primary filings — flagged in confidence. || W1=0: Pure B2B supplier; content within current operator-channel model only | W2=1: Capex into studios/content only, not player-acquisition or AI/wallet bets | W3=1: 800+ supply deals with operators, not demand-reshaping alliances | W4=0: No owned app, wallet, AI assistant, or player-facing surface | W5=0: No owned audience; reaches players only via operator brands | D1=5: Dominant must-have live-casino/RNG content across 800+ operators | D2=1: Content API only; no owned PAM, wallet, or bonusing engine | D3=4: Broad tier-1 supplier licensing; UK licence under active UKGC review | D4=0: No payments or merchant-of-record function; pure content supplier | D5=5: Global reach via 800+ operator brands; record 2025 revenue | D6=3: Trusted live-dealer brand among players; not a wallet destination | AI1=1: No evidence of owning/training models; likely licensed AI tooling | AI2=0: No agentic capability shipped to players | AI3=0: No MCP/A2A/UCP/ACP adoption found | AI4=0: No customer-facing conversational assistant found | AI5=1: Localized/themed content per market; no individual-level personalisation shown | AI6=3: Cross-operator live-dealer behavioral data at scale | AI7=1: AI-tooling consumer (localisation); no platform-for-others position found | F1=5: Profitable, self-funded, no capital constraint evident | F2=5: Record 2025 revenue &gt;EUR2.4bn, ~66% EBITDA margin | F3=5: Cash-generative; indefinite runway as profitable public company | F4=4: Low leverage typical of business model, not independently verified | F5=5: Nasdaq Stockholm listed, ~$13.4bn market cap, broad capital access</t>
+        </is>
+      </c>
+      <c r="DJ9" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="DK9" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="DL9" t="inlineStr">
+        <is>
+          <t>sonnet/company-researcher</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Better Collective A/S</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Copenhagen, Denmark</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>2004</v>
+      </c>
+      <c r="D10" t="n">
+        <v>1900</v>
+      </c>
+      <c r="F10" t="n">
+        <v>800</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Affiliate &amp; media</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Sports-media/affiliate group monetizing via CPA and revenue-share deals with sportsbooks plus a Paid Media (bought-traffic) segment; new Playbook AI betslip product adds an owned engagement layer.</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>B2C sports-media audience, monetized B2B2C via sportsbook revenue-share deals</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>Playbook built on external AI models for bet-slip image recognition and generation</t>
+        </is>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>First-party betting-intent engagement data across a large media network</t>
+        </is>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>X (Twitter) — Playbook named official/exclusive global betting product</t>
+        </is>
+      </c>
+      <c r="AF10" t="inlineStr">
+        <is>
+          <t>X/Twitter (exclusive global AI-betting partner for Playbook); Playmaker Capital, RotoGrinders, Playmaker HQ (acquisitions among 30 total)</t>
+        </is>
+      </c>
+      <c r="AM10" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AN10" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AO10" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AP10" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AQ10" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AR10" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AS10" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AT10" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AV10" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AX10" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AZ10" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="BB10" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="BD10" t="n">
+        <v>1</v>
+      </c>
+      <c r="BI10" t="n">
+        <v>4</v>
+      </c>
+      <c r="BJ10" t="n">
+        <v>3</v>
+      </c>
+      <c r="BK10" t="n">
+        <v>4</v>
+      </c>
+      <c r="BL10" t="n">
+        <v>4</v>
+      </c>
+      <c r="BM10" t="n">
+        <v>4</v>
+      </c>
+      <c r="BN10" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP10" t="n">
+        <v>1</v>
+      </c>
+      <c r="BQ10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BR10" t="n">
+        <v>4</v>
+      </c>
+      <c r="BS10" t="n">
+        <v>2</v>
+      </c>
+      <c r="BT10" t="n">
+        <v>2</v>
+      </c>
+      <c r="BU10" t="n">
+        <v>2</v>
+      </c>
+      <c r="BV10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW10" t="n">
+        <v>3</v>
+      </c>
+      <c r="BX10" t="n">
+        <v>2</v>
+      </c>
+      <c r="BY10" t="n">
+        <v>3</v>
+      </c>
+      <c r="BZ10" t="n">
+        <v>3</v>
+      </c>
+      <c r="CA10" t="n">
+        <v>75</v>
+      </c>
+      <c r="CB10" t="n">
+        <v>20</v>
+      </c>
+      <c r="CC10" t="n">
+        <v>40</v>
+      </c>
+      <c r="CD10" t="n">
+        <v>30</v>
+      </c>
+      <c r="CE10" t="n">
+        <v>48</v>
+      </c>
+      <c r="CF10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="CG10" t="inlineStr">
+        <is>
+          <t>Aspirant</t>
+        </is>
+      </c>
+      <c r="CH10" t="inlineStr">
+        <is>
+          <t>No licence, wallet, or product (odds/games) of its own — still depends on operator partners</t>
+        </is>
+      </c>
+      <c r="CJ10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="CK10" t="inlineStr">
+        <is>
+          <t>0-12m</t>
+        </is>
+      </c>
+      <c r="CL10" t="inlineStr">
+        <is>
+          <t>Turns affiliate traffic into an AI-native, higher-margin acquisition rail incumbents still need</t>
+        </is>
+      </c>
+      <c r="CN10" t="inlineStr">
+        <is>
+          <t>Legal entity Better Collective A/S, listed Nasdaq Copenhagen/Stockholm (BETCO). Playbook is delivered as a product on X's platform (partner-dependent distribution), not a fully independent owned surface — tempers the direct_channel read to 'y with caveat'.</t>
+        </is>
+      </c>
+      <c r="CQ10" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="CU10" t="inlineStr">
+        <is>
+          <t>FY2025 guidance EUR320-350M revenue; Q1 2026 revenue EUR86.3M, +5% YoY organic</t>
+        </is>
+      </c>
+      <c r="CY10" t="n">
+        <v>4</v>
+      </c>
+      <c r="CZ10" t="n">
+        <v>4</v>
+      </c>
+      <c r="DA10" t="n">
+        <v>4</v>
+      </c>
+      <c r="DB10" t="n">
+        <v>2</v>
+      </c>
+      <c r="DC10" t="n">
+        <v>4</v>
+      </c>
+      <c r="DD10" t="n">
+        <v>72</v>
+      </c>
+      <c r="DE10" t="inlineStr">
+        <is>
+          <t>Stable</t>
+        </is>
+      </c>
+      <c r="DH10" t="inlineStr">
+        <is>
+          <t>https://next.io/news/results/q126-revenue-growth-better-collective-in-black/ ; https://www.gamblingnews.com/news/better-collective-posts-q1-growth-maintains-2026-outlook/ ; https://www.intergameonline.com/igaming/news/better-collective-launches-playbook-on-x ; https://tracxn.com/d/acquisitions/acquisitions-by-better-collective/__4BVerZTj81yfPXpgzx86gLvlxeJhuzuHPS6QQQoGBIQ</t>
+        </is>
+      </c>
+      <c r="DI10" t="inlineStr">
+        <is>
+          <t>Strong recent evidence: Q1 2026 report (May 2026), multiple trade-press pieces on the Playbook/X launch (Sept 2025) and its global expansion (May 2026). Two WebFetch attempts on primary trade-press pages returned 403; relied on WebSearch summaries of the same stories from multiple outlets for corroboration. || W1=4: Positions Playbook to bypass Google/affiliate-SEO acquisition directly | W2=3: Steady M&amp;A (30 deals) plus fresh strategic bet on AI product Playbook | W3=4: Exclusive global 'official betting partner' deal with X | W4=4: Playbook AI betslip tool live, expanding into new markets | W5=4: Owns large sports-media/tipster network drawing direct betting-intent traffic | D1=1: No own odds/markets; aggregates and links to third-party sportsbooks | D2=0: No PAM, wallet, or trading/risk infrastructure of its own | D3=1: Media/affiliate registrations only; not a licensed gambling operator | D4=0: No payments or merchant-of-record capability | D5=4: Media network across 20+ regulated markets, ~EUR320-350M revenue | D6=2: Respected sports-media/tipster brand; not a deposit-taking betting brand | AI1=2: Playbook built on external AI models, no own foundation model | AI2=2: Assistive betslip generation with deep-links, not autonomous placement | AI3=0: No MCP/A2A/UCP/ACP adoption found | AI4=3: Playbook is primary AI interface for bet content on X | AI5=2: Segment-level content targeting; no individual AI personalisation evidenced | AI6=3: Large first-party betting-intent engagement dataset across media network | AI7=3: Exclusive AI-betting-partner status on X is a real platform position | F1=4: Profitable public company, self-funded, some debt from M&amp;A history | F2=4: EBITDA guide EUR100-120M on EUR320-350M revenue; net profit in Q1 | F3=4: Ongoing profitable operations support runway | F4=2: Aggressive debt-funded M&amp;A history (30 deals); leverage not independently verified | F5=4: Nasdaq-listed, ~$0.8bn market cap, moderate capital access</t>
+        </is>
+      </c>
+      <c r="DJ10" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="DK10" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="DL10" t="inlineStr">
+        <is>
+          <t>sonnet/company-researcher</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Polymarket</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>New York, USA</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>2020</v>
+      </c>
+      <c r="D11" t="n">
+        <v>423</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1805</v>
+      </c>
+      <c r="F11" t="n">
+        <v>15000</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>AI-native &amp; prediction markets</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Crypto-native (USDC/pUSD) event-contract exchange; earns trading/spread revenue on volume, now operating a CFTC-regulated US arm (Polymarket US via QCX LLC) alongside its international crypto platform.</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>B2C global retail traders plus growing institutional flow; US arm now a regulated exchange</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t>L0</t>
+        </is>
+      </c>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>Real-time crowd-priced probabilities widely cited by media/forecasters as a benchmark</t>
+        </is>
+      </c>
+      <c r="AF11" t="inlineStr">
+        <is>
+          <t>ICE/Intercontinental Exchange (investor, $2bn+ committed); Nasdaq Private Market (resolution-data partner for private-company markets); MLS (sports data/promo partnership)</t>
+        </is>
+      </c>
+      <c r="AH11" t="inlineStr">
+        <is>
+          <t>CFTC-regulated exchange/clearinghouse in the US (via QCX LLC / Polymarket US, since Sept 2025); grey/unlicensed as a gambling product in most other jurisdictions</t>
+        </is>
+      </c>
+      <c r="AL11" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AM11" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AN11" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AO11" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AP11" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AQ11" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AR11" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AS11" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AT11" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AV11" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AX11" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AZ11" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="BB11" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="BD11" t="n">
+        <v>2</v>
+      </c>
+      <c r="BI11" t="n">
+        <v>4</v>
+      </c>
+      <c r="BJ11" t="n">
+        <v>5</v>
+      </c>
+      <c r="BK11" t="n">
+        <v>4</v>
+      </c>
+      <c r="BL11" t="n">
+        <v>5</v>
+      </c>
+      <c r="BM11" t="n">
+        <v>5</v>
+      </c>
+      <c r="BN11" t="n">
+        <v>3</v>
+      </c>
+      <c r="BO11" t="n">
+        <v>4</v>
+      </c>
+      <c r="BP11" t="n">
+        <v>3</v>
+      </c>
+      <c r="BQ11" t="n">
+        <v>3</v>
+      </c>
+      <c r="BR11" t="n">
+        <v>4</v>
+      </c>
+      <c r="BS11" t="n">
+        <v>3</v>
+      </c>
+      <c r="BT11" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU11" t="n">
+        <v>1</v>
+      </c>
+      <c r="BV11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BY11" t="n">
+        <v>4</v>
+      </c>
+      <c r="BZ11" t="n">
+        <v>3</v>
+      </c>
+      <c r="CA11" t="n">
+        <v>91</v>
+      </c>
+      <c r="CB11" t="n">
+        <v>67</v>
+      </c>
+      <c r="CC11" t="n">
+        <v>24</v>
+      </c>
+      <c r="CD11" t="n">
+        <v>46</v>
+      </c>
+      <c r="CE11" t="n">
+        <v>64</v>
+      </c>
+      <c r="CF11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="CG11" t="inlineStr">
+        <is>
+          <t>Aspirant</t>
+        </is>
+      </c>
+      <c r="CH11" t="inlineStr">
+        <is>
+          <t>Sports event-contract product still nascent/pending further CFTC approval (parlay-style contracts, FCM licence); not yet a casino or poker substitute</t>
+        </is>
+      </c>
+      <c r="CJ11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="CK11" t="inlineStr">
+        <is>
+          <t>0-12m</t>
+        </is>
+      </c>
+      <c r="CL11" t="inlineStr">
+        <is>
+          <t>Offers a federally-regulated, exchange-based alternative that could pull sports bettors outside the licensed operator/affiliate model entirely</t>
+        </is>
+      </c>
+      <c r="CN11" t="inlineStr">
+        <is>
+          <t>US-regulated operations run through a distinct related entity structure — Polymarket US / QCX LLC (clearing, acquired mid-2025) plus Coming Home GBA LLC (FCM licence applicant) — flagged as related entities, not duplicates, of the core Polymarket brand. Sector tag 'AI-native &amp; prediction markets' reflects the disruption-frame taxonomy, but direct evidence of Polymarket itself building or deploying AI is thin (it is fundamentally exchange/clearing infrastructure, not an AI company) — the AI scores here come out lower than the seedlist's provisional 'mid-high AI' expectation; worth flagging when anchors.md is finalized. By contrast W and D evidence is very strong and recent.</t>
+        </is>
+      </c>
+      <c r="CQ11" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="CU11" t="inlineStr">
+        <is>
+          <t>Annualized revenue crossed $1B in June 2026, six weeks after CFTC-regulated US launch</t>
+        </is>
+      </c>
+      <c r="CY11" t="n">
+        <v>5</v>
+      </c>
+      <c r="CZ11" t="n">
+        <v>3</v>
+      </c>
+      <c r="DA11" t="n">
+        <v>5</v>
+      </c>
+      <c r="DC11" t="n">
+        <v>5</v>
+      </c>
+      <c r="DD11" t="n">
+        <v>90</v>
+      </c>
+      <c r="DE11" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="DH11" t="inlineStr">
+        <is>
+          <t>https://ir.theice.com/press/news-details/2026/Intercontinental-Exchange-Announces-New-600-Million-Investment-in-Polymarket/default.aspx ; https://www.cnbc.com/2026/06/26/polymarket-annualized-revenue-1-billion-us-exchange-.html ; https://www.covers.com/industry/polymarket-files-parlay-style-sports-contracts-with-cftc-may-21-2026 ; https://www.cnbc.com/2026/05/19/polymarket-launches-private-company-trading-so-investors-can-speculate-on-anthropic-openai.html ; https://docs.polymarket.com/polymarket-learn/FAQ/is-my-money-safe ; https://startpolymarket.com/guides/how-to-deposit/</t>
+        </is>
+      </c>
+      <c r="DI11" t="inlineStr">
+        <is>
+          <t>Very strong, very recent (2026) evidence: CFTC-regulated US launch, ICE investment tranches (Oct 2025 + Mar 2026), Q1 2026 volume and June 2026 revenue milestone, May 2026 CFTC sports-contract filing, May 2026 Nasdaq Private Market partnership. || W1=4: Positions as CFTC-regulated alternative to licensed sportsbooks/affiliates | W2=5: Raised $2bn+ from ICE, acquired QCEX exchange/clearing infra directly | W3=4: ICE strategic investment plus MLS deal reposition sports-funnel access | W4=5: Full-featured trading app live; US-regulated app launched May 2026 | W5=5: Owns intent directly; $26bn Q1 2026 volume on its own platform | D1=3: Broad self-created markets, but sports/casino verticals still nascent | D2=4: Proven owned exchange/clearing (QCEX) handling billions in volume | D3=3: CFTC-regulated in the US; grey/unlicensed as gambling elsewhere | D4=3: US app supports ACH/card/Apple Pay; international remains crypto-only | D5=4: Global reach, tens of billions in quarterly volume, active users undisclosed | D6=3: High-profile brand; regulatory scrutiny/investigation reports persist | AI1=1: No evidence Polymarket trains or fine-tunes its own AI models | AI2=1: Third-party bots trade via public API; no official Polymarket agent shipped | AI3=0: Public API enables unofficial community MCP wrappers, not formal adoption | AI4=0: No official customer-facing AI assistant found | AI5=0: No evidence of AI-driven personalisation of markets or offers | AI6=4: Crowd-priced probabilities widely cited as a forecasting benchmark | AI7=3: Forecasting tools/AI agents consume Polymarket data as ground truth | F1=5: $2bn+ raised from ICE alone; extremely well capitalised | F2=3: $1bn annualized revenue (Jun 2026); net profitability undisclosed | F3=5: $1.8bn+ raised plus fast-ramping revenue implies long runway | F4=None: Private company; leverage/debt data not disclosed | F5=5: ICE-backed, pursuing $15bn valuation round, excellent capital access</t>
+        </is>
+      </c>
+      <c r="DJ11" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="DK11" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="DL11" t="inlineStr">
+        <is>
+          <t>sonnet/company-researcher</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Rithmm, Inc.</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Chestnut Hill, MA, USA</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>2022</v>
+      </c>
+      <c r="E12" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>AI-native &amp; prediction markets</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Consumer subscription app (~$30/month) offering AI-built predictive models for player props, game picks, parlays and DFS lineups; analytics-only, does not take wagers itself.</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>B2C — individual US sports bettors and DFS players</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>Appears to build on external AI/LLM APIs for its 'AI builds a model for you' feature; specific vendor unconfirmed</t>
+        </is>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AA12" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t>None evident beyond licensed/public sports data feeds</t>
+        </is>
+      </c>
+      <c r="AL12" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AM12" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AN12" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AO12" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AP12" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AQ12" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AR12" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AS12" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AT12" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AV12" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AX12" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AZ12" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="BB12" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="BD12" t="n">
+        <v>1</v>
+      </c>
+      <c r="BI12" t="n">
+        <v>1</v>
+      </c>
+      <c r="BJ12" t="n">
+        <v>2</v>
+      </c>
+      <c r="BK12" t="n">
+        <v>1</v>
+      </c>
+      <c r="BL12" t="n">
+        <v>3</v>
+      </c>
+      <c r="BM12" t="n">
+        <v>2</v>
+      </c>
+      <c r="BN12" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO12" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP12" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ12" t="n">
+        <v>0</v>
+      </c>
+      <c r="BR12" t="n">
+        <v>1</v>
+      </c>
+      <c r="BS12" t="n">
+        <v>2</v>
+      </c>
+      <c r="BT12" t="n">
+        <v>2</v>
+      </c>
+      <c r="BU12" t="n">
+        <v>1</v>
+      </c>
+      <c r="BV12" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW12" t="n">
+        <v>3</v>
+      </c>
+      <c r="BX12" t="n">
+        <v>4</v>
+      </c>
+      <c r="BY12" t="n">
+        <v>1</v>
+      </c>
+      <c r="BZ12" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA12" t="n">
+        <v>35</v>
+      </c>
+      <c r="CB12" t="n">
+        <v>11</v>
+      </c>
+      <c r="CC12" t="n">
+        <v>30</v>
+      </c>
+      <c r="CD12" t="n">
+        <v>20</v>
+      </c>
+      <c r="CE12" t="n">
+        <v>26</v>
+      </c>
+      <c r="CF12" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="CG12" t="inlineStr">
+        <is>
+          <t>Dormant</t>
+        </is>
+      </c>
+      <c r="CH12" t="inlineStr">
+        <is>
+          <t>No owned odds/content, no gambling licence, minimal distribution scale versus well-funded rivals (PrizePicks, Underdog)</t>
+        </is>
+      </c>
+      <c r="CJ12" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="CK12" t="inlineStr">
+        <is>
+          <t>3y+</t>
+        </is>
+      </c>
+      <c r="CL12" t="inlineStr">
+        <is>
+          <t>Marginal on its own; a small analytics layer that still funnels bettors to incumbent sportsbooks</t>
+        </is>
+      </c>
+      <c r="CN12" t="inlineStr">
+        <is>
+          <t>Founded 2022 by CEO Megan Lanham and CTO Brian Beachkofski. This is the seedlist's designated low-end 'dormant' calibration anchor, and the evidence supports that: no press coverage found in the last 18 months, only one confirmed funding round ($2M seed, May 2023; $4.5M across 2 rounds total per Tracxn, unverified beyond that), no official IR/press presence. No subsidiary/duplicate concerns — small standalone entity.</t>
+        </is>
+      </c>
+      <c r="CQ12" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="CY12" t="n">
+        <v>2</v>
+      </c>
+      <c r="DC12" t="n">
+        <v>1</v>
+      </c>
+      <c r="DD12" t="n">
+        <v>30</v>
+      </c>
+      <c r="DE12" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="DH12" t="inlineStr">
+        <is>
+          <t>https://tracxn.com/d/companies/rithmm/__fV5H_jH0k275_d-xd9hlK3tWIa2HcIgBEATcAvi9w3k ; https://apps.apple.com/us/app/rithmm-ai-sports-betting/id1641010681 ; https://www.rithmm.com/post/ai-tools-for-sports-betting ; https://picksandparlays.net/reviews/ai-picks/rithmm</t>
+        </is>
+      </c>
+      <c r="DI12" t="inlineStr">
+        <is>
+          <t>Weak evidence tier throughout: app-store listings, review/aggregator sites, and a funding aggregator (Tracxn) — no primary-source press, filings, or company disclosures found in the last 18 months. Treat all scores here as best-effort inference, not confirmed fact. || W1=1: No channel-bypass stance found; complements existing sportsbooks | W2=2: One AI-focused seed raise ($4.5M); no further funding/M&amp;A found | W3=1: Integrates odds comparisons across books; no major alliances found | W4=3: AI model-builder app shipped and live on iOS/Android | W5=2: Modest but real subscriber base (4.4/5 rating, 1,400+ reviews) | D1=1: No own odds/content; aggregates third-party sportsbook lines | D2=0: No PAM, wallet, or trading-rail infrastructure of its own | D3=0: Analytics-only; not a licensed gambling entity | D4=0: Subscription billing only via app stores, no gambling MoR | D5=1: Niche US-focused subscriber base, small single-market scale | D6=2: Positive niche reputation, limited broad market awareness | AI1=2: Model-generation feature likely built on external AI/LLM APIs | AI2=1: Assistive AI model-builder only, no autonomous bet placement | AI3=0: No MCP/A2A/UCP/ACP adoption found | AI4=3: In-app 'ask AI to build a model' functions as a shipped assistant | AI5=4: User-customizable weighted AI models are the core product | AI6=1: Likely licensed/public sports data feeds, no unique data moat | AI7=0: Consumer of external AI/data services; no ecosystem-platform position | F1=2: $4.5M total raised across 2 rounds, modest for scaling ambitions | F2=None: Private; no revenue/profitability disclosed | F3=None: Last disclosed raise 2023; current runway unknown | F4=None: Private; no debt/leverage data available | F5=1: Thin funding history; no recent capital raise found</t>
+        </is>
+      </c>
+      <c r="DJ12" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="DK12" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="DL12" t="inlineStr">
+        <is>
+          <t>sonnet/company-researcher</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Sportradar Group AG</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>St. Gallen, Switzerland</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>2001</v>
+      </c>
+      <c r="D13" t="n">
+        <v>4582</v>
+      </c>
+      <c r="F13" t="n">
+        <v>4520</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Data &amp; odds</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>B2B sports-data, odds/trading, integrity and ad-tech provider to betting operators, leagues and media; now extending into prediction-market exchanges. Monetizes via data/technology licensing and managed trading services fees.</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>B2B — betting operators, sports leagues, media, and (new) prediction-market exchanges</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>Trains its own proprietary generative basketball foundation model (body-pose data, billions of datapoints); soccer/tennis planned to follow</t>
+        </is>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AA13" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>Official league data rights plus computer-vision tracking across major sports</t>
+        </is>
+      </c>
+      <c r="AF13" t="inlineStr">
+        <is>
+          <t>Kalshi (multi-year global data/infrastructure partnership, June 2026); IMG Arena/Endeavor rights portfolio acquired Nov 2025 (Wimbledon, PGA Tour, EuroLeague, WTA, MLS); MLB, NHL, UFC rights deals</t>
+        </is>
+      </c>
+      <c r="AH13" t="inlineStr">
+        <is>
+          <t>56+ North American supplier licences (states/tribes/Canada); UK Gambling Commission licensed; UAE GCGRA vendor licence</t>
+        </is>
+      </c>
+      <c r="AK13" t="inlineStr">
+        <is>
+          <t>Bettor Sense AI responsible-gambling product live/in-trial with 13+ operators, ~6M player accounts profiled in 2025</t>
+        </is>
+      </c>
+      <c r="AM13" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AN13" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AO13" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AP13" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AQ13" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AR13" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AS13" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AT13" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AV13" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AX13" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AZ13" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="BB13" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="BD13" t="n">
+        <v>1</v>
+      </c>
+      <c r="BI13" t="n">
+        <v>2</v>
+      </c>
+      <c r="BJ13" t="n">
+        <v>4</v>
+      </c>
+      <c r="BK13" t="n">
+        <v>4</v>
+      </c>
+      <c r="BL13" t="n">
+        <v>2</v>
+      </c>
+      <c r="BM13" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN13" t="n">
+        <v>5</v>
+      </c>
+      <c r="BO13" t="n">
+        <v>4</v>
+      </c>
+      <c r="BP13" t="n">
+        <v>5</v>
+      </c>
+      <c r="BQ13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BR13" t="n">
+        <v>5</v>
+      </c>
+      <c r="BS13" t="n">
+        <v>1</v>
+      </c>
+      <c r="BT13" t="n">
+        <v>4</v>
+      </c>
+      <c r="BU13" t="n">
+        <v>2</v>
+      </c>
+      <c r="BV13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW13" t="n">
+        <v>2</v>
+      </c>
+      <c r="BX13" t="n">
+        <v>3</v>
+      </c>
+      <c r="BY13" t="n">
+        <v>5</v>
+      </c>
+      <c r="BZ13" t="n">
+        <v>4</v>
+      </c>
+      <c r="CA13" t="n">
+        <v>56</v>
+      </c>
+      <c r="CB13" t="n">
+        <v>72</v>
+      </c>
+      <c r="CC13" t="n">
+        <v>55</v>
+      </c>
+      <c r="CD13" t="n">
+        <v>64</v>
+      </c>
+      <c r="CE13" t="n">
+        <v>61</v>
+      </c>
+      <c r="CF13" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="CG13" t="inlineStr">
+        <is>
+          <t>Sleeping giant</t>
+        </is>
+      </c>
+      <c r="CH13" t="inlineStr">
+        <is>
+          <t>No owned consumer distribution or wallet; value capture stays entirely B2B</t>
+        </is>
+      </c>
+      <c r="CJ13" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="CK13" t="inlineStr">
+        <is>
+          <t>1-3y</t>
+        </is>
+      </c>
+      <c r="CL13" t="inlineStr">
+        <is>
+          <t>Extends its rail-beneath-the-rails power into prediction markets too, deepening incumbent dependency on it</t>
+        </is>
+      </c>
+      <c r="CN13" t="inlineStr">
+        <is>
+          <t>Legal entity Sportradar Group AG (Swiss-domiciled), NASDAQ: SRAD. IMG ARENA acquisition closed Nov 2025, structured at no net cash cost to Sportradar. Distinct company from competitor Genius Sports — not a duplicate or subsidiary relationship.</t>
+        </is>
+      </c>
+      <c r="CQ13" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="CU13" t="inlineStr">
+        <is>
+          <t>2026 guidance EUR1,557-1,582M revenue, 23-25% constant-currency growth; Q1 2026 revenue EUR347M (+11% YoY)</t>
+        </is>
+      </c>
+      <c r="CY13" t="n">
+        <v>4</v>
+      </c>
+      <c r="CZ13" t="n">
+        <v>3</v>
+      </c>
+      <c r="DA13" t="n">
+        <v>4</v>
+      </c>
+      <c r="DB13" t="n">
+        <v>3</v>
+      </c>
+      <c r="DC13" t="n">
+        <v>4</v>
+      </c>
+      <c r="DD13" t="n">
+        <v>72</v>
+      </c>
+      <c r="DE13" t="inlineStr">
+        <is>
+          <t>Stable</t>
+        </is>
+      </c>
+      <c r="DH13" t="inlineStr">
+        <is>
+          <t>https://sportradar.com/content-hub/news/sportradar-and-kalshi-announce-first-of-its-kind-data-and-infrastructure-global-partnership-for-prediction-markets/?lang=en-us ; https://investors.sportradar.com/news-releases/news-release-details/sportradar-announces-close-acquisition-img-arena-and-its ; https://www.casino.org/news/sportradar-most-ai-advanced-gaming-company-says-analyst/ ; https://sportradar.com/integrity-regulatory/regulatory-services/bettor-sense/?lang=en-us ; https://companiesmarketcap.com/sportradar/marketcap/</t>
+        </is>
+      </c>
+      <c r="DI13" t="inlineStr">
+        <is>
+          <t>Strong, recent (2025-2026) evidence: SEC 6-K filings, investor-day AI demonstrations, the Kalshi partnership press release (June 2026), and a Jefferies analyst note (June 2025) rating it the most AI-advanced company in gaming. || W1=2: Extends B2B data supply to new customer types, not direct-to-player | W2=4: IMG Arena acquisition plus Kalshi deal plus AI investor day | W3=4: Landmark Kalshi partnership plus major league rights reposition funnel | W4=2: Bettor Sense/Bet Concierge shipped but delivered via operators only | W5=1: No owned consumer audience; reaches players via operators/media only | D1=5: Official data/odds rights across major leagues, must-have supply position | D2=4: Managed Trading Services provide real pricing/risk infrastructure | D3=5: 56+ NA licences, UK/UAE licensed, dedicated integrity/regulatory division | D4=0: No payments or merchant-of-record function | D5=5: Global supplier, EUR1.56-1.58bn 2026 revenue guide, ~5,000 staff | D6=1: Industry-recognized supplier brand, largely invisible to end bettors | AI1=4: Trained proprietary generative basketball foundation model on billions of datapoints | AI2=2: Bet Concierge chatbot prototyping bet-building, not yet broad production | AI3=0: No MCP/A2A/UCP/ACP adoption found | AI4=2: Bet Concierge/Bettor Sense chatbots exist, delivered via operator apps | AI5=3: GenAI audio plus personalized odds/content described at segment level | AI6=5: Official rights plus computer-vision tracking, industry-defining data moat | AI7=4: Analyst-rated most AI-advanced in sector; leagues/exchanges build on its data | F1=4: Well-capitalised public company, ~$4.5bn market cap | F2=3: Strong revenue growth (23-25%) but reported net loss in Q1 2026 | F3=4: Growing revenue, public company, no near-term runway concern | F4=3: IMG Arena deal structured with no cash outlay; leverage unverified | F5=4: Nasdaq-listed, demonstrated M&amp;A capacity via deal structuring</t>
+        </is>
+      </c>
+      <c r="DJ13" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="DK13" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="DL13" t="inlineStr">
+        <is>
+          <t>sonnet/company-researcher</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Rescue 4 companies from the killed batch-02 run (crash-safety proven)
The batch-02 fleet died again - this time on a monthly spend limit - but the
new incremental-write design meant the research was NOT lost:

- 4 companies (Kaizen Gaming, Genius Sports, Catena Media, Trustly) had already
  been written to batches/raw/ by the agents mid-run and were recovered with
  `populate.py igaming --from-raw`. Under the old design these would have been
  zero, as in the two previous kills.
- Workbook now 14 companies; qa_check: 10 passed, 0 warnings, 0 failures;
  calibration anchors stable.
- Consumed raw files retired to raw/consumed/ as the audit trail.

PROGRESS.md now carries a blocker notice: the monthly spend limit stops further
research agents until it is raised or resets. 11 companies remain from batch 02.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/industries/igaming/igaming_landscape.xlsx
+++ b/industries/igaming/igaming_landscape.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DL13"/>
+  <dimension ref="A1:DL17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4603,6 +4603,1308 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Catena Media plc</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Malta (listed Nasdaq Stockholm)</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>2012</v>
+      </c>
+      <c r="F14" t="n">
+        <v>27</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Affiliate &amp; media</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>SEO/content and paid-media affiliate marketing for sports betting and casino, monetized via CPA/revenue-share deals with operators; recently diversifying into sub-affiliation network fees (MRKTPLAYS/MRKTPLAYS+) and paid media/CRM channels beyond organic search.</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>B2B/B2B2C: sells player leads and traffic to licensed operators; North America (98% of group revenue) is now the core geography</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>Built and then discontinued a JV generative-AI content-production tool (MVP Feb 2024, JV wound down/bought out Jan 2025, recovering EUR 0.7m of the investment, EUR 1.2m impairment); AI now framed as a general content/scaling enhancer, not a proprietary model effort</t>
+        </is>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AA14" t="inlineStr">
+        <is>
+          <t>L0</t>
+        </is>
+      </c>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t>Former specialist-AI JV partner for content generation (name not disclosed, venture discontinued Jan 2025); no current disclosed gen-AI platform partnership</t>
+        </is>
+      </c>
+      <c r="AF14" t="inlineStr">
+        <is>
+          <t>Operator commission/CPA partners across NA sportsbook and casino brands; MRKTPLAYS+ sub-affiliate/publisher partners (working-capital and minority-equity participation offered to partners)</t>
+        </is>
+      </c>
+      <c r="AM14" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AN14" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AO14" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AP14" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AQ14" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AR14" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AS14" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AT14" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AV14" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AX14" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AZ14" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="BB14" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="BD14" t="n">
+        <v>2</v>
+      </c>
+      <c r="BI14" t="n">
+        <v>3</v>
+      </c>
+      <c r="BJ14" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK14" t="n">
+        <v>2</v>
+      </c>
+      <c r="BL14" t="n">
+        <v>2</v>
+      </c>
+      <c r="BM14" t="n">
+        <v>2</v>
+      </c>
+      <c r="BN14" t="n">
+        <v>3</v>
+      </c>
+      <c r="BO14" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP14" t="n">
+        <v>1</v>
+      </c>
+      <c r="BQ14" t="n">
+        <v>0</v>
+      </c>
+      <c r="BR14" t="n">
+        <v>3</v>
+      </c>
+      <c r="BS14" t="n">
+        <v>2</v>
+      </c>
+      <c r="BT14" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU14" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV14" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW14" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX14" t="n">
+        <v>2</v>
+      </c>
+      <c r="BY14" t="n">
+        <v>2</v>
+      </c>
+      <c r="BZ14" t="n">
+        <v>1</v>
+      </c>
+      <c r="CA14" t="n">
+        <v>40</v>
+      </c>
+      <c r="CB14" t="n">
+        <v>33</v>
+      </c>
+      <c r="CC14" t="n">
+        <v>15</v>
+      </c>
+      <c r="CD14" t="n">
+        <v>24</v>
+      </c>
+      <c r="CE14" t="n">
+        <v>30</v>
+      </c>
+      <c r="CF14" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="CG14" t="inlineStr">
+        <is>
+          <t>Dormant</t>
+        </is>
+      </c>
+      <c r="CH14" t="inlineStr">
+        <is>
+          <t>No licence, betting product, or payments/MoR capability; its AI investment record (one JV, discontinued in ~a year) is thin, and its core organic-search channel is the one AI answer engines are actively eating.</t>
+        </is>
+      </c>
+      <c r="CJ14" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="CK14" t="inlineStr">
+        <is>
+          <t>1-3y</t>
+        </is>
+      </c>
+      <c r="CL14" t="inlineStr">
+        <is>
+          <t>Willing but structurally unable: the clearest 'affiliate under AI-search attack' case in the set — explicitly reshaping itself around AI disruption of its own channel, but has no licence, product or wallet and its own AI content bet already failed.</t>
+        </is>
+      </c>
+      <c r="CN14" t="inlineStr">
+        <is>
+          <t>Legal entity Catena Media plc, Malta-incorporated, Nasdaq Stockholm-listed (CTM). Divested esports assets (esports.net, esportsbet.com) in Q2 2025 and cut headcount ~25% in a 2025 rightsizing; now near-exclusively a North America sports betting/casino affiliate business (98% of revenue). Market cap conflicting across sources (SEK 187.99m per stockanalysis.com mid-June 2026 vs SEK 278.39m at a more recent date) — reported ~USD 27m using an approx. 10.4 SEK/USD rate; treat as directional, not precise.</t>
+        </is>
+      </c>
+      <c r="CQ14" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="CU14" t="inlineStr">
+        <is>
+          <t>Q1 2026 revenue EUR 12.3m (+26% YoY); Q4 2025 revenue EUR 15.6m (+53% YoY), adj. EBITDA EUR 4.7m; North America ~98% of group revenue by year-end 2025</t>
+        </is>
+      </c>
+      <c r="CY14" t="n">
+        <v>2</v>
+      </c>
+      <c r="CZ14" t="n">
+        <v>2</v>
+      </c>
+      <c r="DA14" t="n">
+        <v>3</v>
+      </c>
+      <c r="DB14" t="n">
+        <v>4</v>
+      </c>
+      <c r="DC14" t="n">
+        <v>2</v>
+      </c>
+      <c r="DD14" t="n">
+        <v>52</v>
+      </c>
+      <c r="DE14" t="inlineStr">
+        <is>
+          <t>At-risk</t>
+        </is>
+      </c>
+      <c r="DH14" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/strength-in-north-america-delivers-revenue-growth-as-new-strategic-focus-takes-root-catena-media-301752711.html ; https://www.investing.com/news/transcripts/earnings-call-transcript-catena-media-sees-q1-2026-revenue-rise-26-stock-jumps-93CH-4681653 ; https://sbcamericas.com/2025/02/11/catena-media-q4-earnings-ai-deal/ ; https://www.igbaffiliate.com/en/articles/119738/catena-dumps-ai-plan-while-fy24-revenue-slumps-35/ ; https://sbcamericas.com/2025/09/19/catena-media-launches-mrktplays/ ; https://stockanalysis.com/quote/sto/CTM/market-cap/ ; https://next.io/news/people/catena-kindred-veteran-manuel-stan-ceo/</t>
+        </is>
+      </c>
+      <c r="DI14" t="inlineStr">
+        <is>
+          <t>Financials well documented via own investor releases and trade press through Q1 2026. Strategic/AI commentary from CEO Manuel Stan corroborated across multiple outlets, though the fullest interview (EGR) is paywalled so only headline framing could be captured, not direct quotes. || W1=3: CEO says AI is 'uprooting' affiliate model; must become direct destination | W2=1: Discontinued its only AI bet (content-gen JV) after ~1 year | W3=2: Operator CPA deals plus new sub-affiliate network partners only | W4=2: MRKTPLAYS/MRKTPLAYS+ sub-affiliation platform shipped; AI content tool failed/closed | W5=2: Owns SEO/organic intent traffic, but CTR collapsing under AI Overviews | D1=3: Aggregates odds/offers content only; no owned betting product | D2=1: No PAM/wallet/trading rail; pure marketing/lead-gen tech stack | D3=1: No gambling licence itself; media/marketing entity only | D4=0: No payments or MoR role; monetized via operator commissions | D5=3: North America-focused (98% of revenue); narrowed from prior global footprint | D6=2: Recognized affiliate brand in NA niche, not a betting brand players trust with money | AI1=1: Only AI bet (content-gen JV) built then discontinued within a year | AI2=0: No agentic assistant capability shipped or planned found | AI3=0: No MCP/A2A/UCP/ACP adoption evidence found | AI4=0: No customer-facing conversational assistant found | AI5=2: Content/SEO targeting per-segment, not proven individual-level personalization | AI6=2: Deep affiliate-funnel conversion data across NA operators, moderately useful | AI7=1: Pure consumer/failed experimenter of gen-AI tools, not an ecosystem partner | F1=2: Small-cap turnaround story; no fresh funding round found, self-funded from ops | F2=2: Returned to double-digit growth and rising EBITDA margin (22% Q1 2026) after a slump | F3=3: Senior bonds fully redeemed June 2025; leverage target 0-1.75x net debt/EBITDA | F4=4: No outstanding bond debt since June 2025 redemption; low leverage | F5=2: Micro-cap (~SEK 200-280m) with limited public capital-raising leverage</t>
+        </is>
+      </c>
+      <c r="DJ14" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="DK14" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="DL14" t="inlineStr">
+        <is>
+          <t>sonnet/company-researcher</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Genius Sports Limited</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>New York, US / London, UK</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>2001</v>
+      </c>
+      <c r="D15" t="n">
+        <v>2700</v>
+      </c>
+      <c r="F15" t="n">
+        <v>2780</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Data &amp; odds</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Sells official sports data, odds feeds, trading/risk management and AI-driven officiating tech to 300+ sportsbooks and leagues; since April 2026 also owns Legend's affiliate/media network (Covers.com, Casino.org) monetized via advertising and referral commissions.</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>B2B (300+ sportsbooks, leagues, media buyers); newly B2C via Legend's affiliate/media sites</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>Builds proprietary computer-vision / tracking models (GeniusIQ) rather than general-purpose foundation models</t>
+        </is>
+      </c>
+      <c r="Y15" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AA15" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="AC15" t="inlineStr">
+        <is>
+          <t>Official/exclusive data and tracking rights with NFL, NBA, Premier League and 400+ sports bodies; hard to replicate</t>
+        </is>
+      </c>
+      <c r="AF15" t="inlineStr">
+        <is>
+          <t>NFL, NBA, Premier League, CONMEBOL, DraftKings, FanDuel (data supply), Kalshi/prediction-market data, Goldman Sachs and Deutsche Bank (Legend acquisition financing)</t>
+        </is>
+      </c>
+      <c r="AH15" t="inlineStr">
+        <is>
+          <t>US sports-data supplier licences in 11+ states; data/tech operations in 150+ countries (supplier licences, not an operator licence)</t>
+        </is>
+      </c>
+      <c r="AM15" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AN15" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AO15" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AP15" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AQ15" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AR15" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AS15" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AT15" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AV15" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AX15" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AZ15" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="BB15" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="BD15" t="n">
+        <v>3</v>
+      </c>
+      <c r="BI15" t="n">
+        <v>2</v>
+      </c>
+      <c r="BJ15" t="n">
+        <v>4</v>
+      </c>
+      <c r="BK15" t="n">
+        <v>4</v>
+      </c>
+      <c r="BL15" t="n">
+        <v>3</v>
+      </c>
+      <c r="BM15" t="n">
+        <v>4</v>
+      </c>
+      <c r="BN15" t="n">
+        <v>5</v>
+      </c>
+      <c r="BO15" t="n">
+        <v>4</v>
+      </c>
+      <c r="BP15" t="n">
+        <v>2</v>
+      </c>
+      <c r="BQ15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BR15" t="n">
+        <v>4</v>
+      </c>
+      <c r="BS15" t="n">
+        <v>2</v>
+      </c>
+      <c r="BT15" t="n">
+        <v>3</v>
+      </c>
+      <c r="BU15" t="n">
+        <v>2</v>
+      </c>
+      <c r="BV15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX15" t="n">
+        <v>3</v>
+      </c>
+      <c r="BY15" t="n">
+        <v>4</v>
+      </c>
+      <c r="BZ15" t="n">
+        <v>3</v>
+      </c>
+      <c r="CA15" t="n">
+        <v>66</v>
+      </c>
+      <c r="CB15" t="n">
+        <v>63</v>
+      </c>
+      <c r="CC15" t="n">
+        <v>43</v>
+      </c>
+      <c r="CD15" t="n">
+        <v>53</v>
+      </c>
+      <c r="CE15" t="n">
+        <v>58</v>
+      </c>
+      <c r="CF15" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="CG15" t="inlineStr">
+        <is>
+          <t>Aspirant</t>
+        </is>
+      </c>
+      <c r="CH15" t="inlineStr">
+        <is>
+          <t>No wallet, MoR, or betting licence — still needs a licensed money-movement or betting capability to run a transaction end-to-end without an operator.</t>
+        </is>
+      </c>
+      <c r="CJ15" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="CK15" t="inlineStr">
+        <is>
+          <t>0-12m</t>
+        </is>
+      </c>
+      <c r="CL15" t="inlineStr">
+        <is>
+          <t>Bypasses the affiliate rail by owning it: Legend gives Genius 118M+ betting-intent users and a media network operators currently pay to reach, on top of the data feeds books already depend on.</t>
+        </is>
+      </c>
+      <c r="CN15" t="inlineStr">
+        <is>
+          <t>Legal entity Genius Sports Limited (Bermuda-incorporated, NYSE: GENI, went public via SPAC merger with dMY Technology Group VI in 2021). Legend acquisition closed April 2026 for up to $1.2B (Covers.com, Casino.org, Casino Guru among its ~25 brands) — flag as the key driver of this batch's W/D scores; pre-Legend Genius would score materially lower on W4/W5. No subsidiary/duplicate conflicts identified against the existing anchor set.</t>
+        </is>
+      </c>
+      <c r="CQ15" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="CU15" t="inlineStr">
+        <is>
+          <t>FY2025 group revenue $669.5M (+31% YoY); pro forma with Legend, ~$1.1B revenue / $320-330M adj. EBITDA guided for 2026</t>
+        </is>
+      </c>
+      <c r="CY15" t="n">
+        <v>5</v>
+      </c>
+      <c r="CZ15" t="n">
+        <v>4</v>
+      </c>
+      <c r="DA15" t="n">
+        <v>5</v>
+      </c>
+      <c r="DB15" t="n">
+        <v>3</v>
+      </c>
+      <c r="DC15" t="n">
+        <v>5</v>
+      </c>
+      <c r="DD15" t="n">
+        <v>88</v>
+      </c>
+      <c r="DE15" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="DH15" t="inlineStr">
+        <is>
+          <t>https://investors.geniussports.com/news/news-details/2026/Genius-Sports-Reports-Fourth-Quarter-and-Full-Year-2025-Results/default.aspx ; https://www.geniussports.com/newsroom/genius-sports-closes-legend-acquisition-to-expand-media-platform/ ; https://www.affiversemedia.com/genius-sports-acquires-legend-in-1-2-billion-deal-making-it-the-largest-gaming-affiliate-acquisition-ever/ ; https://www.geniussports.com/geniusiq/ ; https://www.theglobeandmail.com/investing/markets/stocks/GENI-N/pressreleases/1664966/genius-sports-closes-legend-acquisition-and-secures-1-05-billion-debt-package/ ; https://www.gamblinginsider.com/news/159115/genius-sports-q1-prediction-markets-legend-beyond-sports-data</t>
+        </is>
+      </c>
+      <c r="DI15" t="inlineStr">
+        <is>
+          <t>Strong recent (2026) primary sources for financials and the Legend deal; AI/agentic-protocol scores are inferential (absence of evidence for MCP/A2A adoption) so overall confidence held at medium rather than high. || W1=2: Core is B2B data vendor; Legend deepens affiliate reach, not overt bypass | W2=4: $1.2B Legend deal, largest gaming-affiliate acquisition ever, major capital shift | W3=4: 300+ sportsbook data deals, league rights, Legend's 25+ affiliate brands | W4=3: FANHub, GeniusIQ AI platform, Legend's consumer sites now live | W5=4: Legend adds 118M unique users / 320M annual visits of betting-intent traffic | D1=5: Official data/odds feeds for NFL, NBA, Premier League and 400+ bodies | D2=4: Genius Trading Services: fully managed odds/risk platform for 300+ books | D3=2: Supplier-level licences in 11+ US states; not a KYC/AML-facing operator | D4=0: No payments or merchant-of-record function; pure data/media business | D5=4: 300+ sportsbook clients, 150+ countries; Legend adds 118M-user audience | D6=2: Known as data/media infrastructure, not a brand players deposit with | AI1=3: Proprietary computer-vision/tracking models (GeniusIQ), not frontier LLMs | AI2=2: SAOT is semi-automated officiating (assistive), not autonomous end-to-end | AI3=0: No evidence of MCP/A2A/UCP/ACP agent-commerce protocol adoption | AI4=0: No public customer-facing conversational assistant found | AI5=3: Moment Engine personalises ads via real-time sports-moment + audience data | AI6=4: Official league data + tracking data forms a genuine, hard-to-copy moat | AI7=3: SAOT/tracking outputs become infrastructure other sports/media firms use | F1=5: Public co., $280.6M cash at YE2025, net-cash position pre-acquisition | F2=4: Adj. EBITDA $136.2M (+59%, 20.4% margin); GAAP net loss on non-cash items | F3=5: Profitable on adj. EBITDA basis with growing cash; runway not a constraint | F4=3: Post-Legend: $825M term loan, net leverage guided &lt;3x, up from near-zero | F5=5: Raised $1.07B debt package from Goldman Sachs/Deutsche Bank readily</t>
+        </is>
+      </c>
+      <c r="DJ15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="DK15" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="DL15" t="inlineStr">
+        <is>
+          <t>sonnet/company-researcher</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Kaizen Gaming International Limited</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Malta (founded Athens, Greece)</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D16" t="n">
+        <v>3000</v>
+      </c>
+      <c r="E16" t="n">
+        <v>74</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Operator (B2C)</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Licensed multi-brand operator monetizing sportsbook/casino margin; Betano is the international brand, Stoiximan the Greece/Cyprus sister brand under a related entity.</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>B2C sports bettors and casino players across 20 regulated markets (Europe, Latin America, Africa)</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>Uses external/partner AI stack (Databricks data platform) plus acquired proprietary sports-trading AI (GameplAI, 2026); no evidence of training own frontier models</t>
+        </is>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AA16" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="AD16" t="inlineStr">
+        <is>
+          <t>Databricks (data/AI infrastructure case study); GameplAI (acquired 2026, AI sports trading and analytics)</t>
+        </is>
+      </c>
+      <c r="AF16" t="inlineStr">
+        <is>
+          <t>Allwyn Entertainment (36.75% minority investor in ex-Greece/Cyprus business), FIFA (global partner), Tottenham Hotspur (sponsorship), GameplAI (acquired 2026), Databricks</t>
+        </is>
+      </c>
+      <c r="AH16" t="inlineStr">
+        <is>
+          <t>20 regulated markets as of 2026 incl. Malta (MGA), Greece, Cyprus, Portugal, Romania, Germany, Brazil, Bulgaria, Czechia, Chile, Peru, Ecuador, Ontario (Canada), Nigeria, Ghana; Spanish general betting licence secured July 2026</t>
+        </is>
+      </c>
+      <c r="AK16" t="inlineStr">
+        <is>
+          <t>In-house AI system 'RG-AID' flags risky play patterns; outputs reviewed by trained RG staff before player-facing action (no fully automated decisions)</t>
+        </is>
+      </c>
+      <c r="AM16" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AN16" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AO16" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AP16" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AQ16" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AR16" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AS16" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AT16" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AV16" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AX16" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AZ16" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="BB16" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="BD16" t="n">
+        <v>3</v>
+      </c>
+      <c r="BI16" t="n">
+        <v>3</v>
+      </c>
+      <c r="BJ16" t="n">
+        <v>3</v>
+      </c>
+      <c r="BK16" t="n">
+        <v>2</v>
+      </c>
+      <c r="BL16" t="n">
+        <v>3</v>
+      </c>
+      <c r="BM16" t="n">
+        <v>2</v>
+      </c>
+      <c r="BN16" t="n">
+        <v>4</v>
+      </c>
+      <c r="BO16" t="n">
+        <v>4</v>
+      </c>
+      <c r="BP16" t="n">
+        <v>4</v>
+      </c>
+      <c r="BQ16" t="n">
+        <v>2</v>
+      </c>
+      <c r="BR16" t="n">
+        <v>4</v>
+      </c>
+      <c r="BS16" t="n">
+        <v>4</v>
+      </c>
+      <c r="BT16" t="n">
+        <v>3</v>
+      </c>
+      <c r="BU16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW16" t="n">
+        <v>1</v>
+      </c>
+      <c r="BX16" t="n">
+        <v>4</v>
+      </c>
+      <c r="BY16" t="n">
+        <v>3</v>
+      </c>
+      <c r="BZ16" t="n">
+        <v>2</v>
+      </c>
+      <c r="CA16" t="n">
+        <v>54</v>
+      </c>
+      <c r="CB16" t="n">
+        <v>74</v>
+      </c>
+      <c r="CC16" t="n">
+        <v>33</v>
+      </c>
+      <c r="CD16" t="n">
+        <v>54</v>
+      </c>
+      <c r="CE16" t="n">
+        <v>54</v>
+      </c>
+      <c r="CF16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="CG16" t="inlineStr">
+        <is>
+          <t>Dormant</t>
+        </is>
+      </c>
+      <c r="CH16" t="inlineStr">
+        <is>
+          <t>No owned discovery/prediction surface, no confirmed merchant-of-record or wallet innovation; audience growth still leans on sponsorship (and likely affiliate) spend rather than owned intent traffic.</t>
+        </is>
+      </c>
+      <c r="CJ16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="CK16" t="inlineStr">
+        <is>
+          <t>1-3y</t>
+        </is>
+      </c>
+      <c r="CL16" t="inlineStr">
+        <is>
+          <t>Strong, fast-expanding operator investing in AI trading and personalization, but still runs the standard licensed-operator acquisition model — incremental modernizer, not a bypass threat.</t>
+        </is>
+      </c>
+      <c r="CN16" t="inlineStr">
+        <is>
+          <t>Legal entity: Kaizen Gaming International Limited (Malta), founded Athens 2012. Betano = international brand; Stoiximan = Greece/Cyprus sister brand under a related entity (different ownership) — not scored here, flag as related but distinct P&amp;L. Allwyn Entertainment holds 36.75% of the ex-Greece/Cyprus business (~EUR 74.2m, Dec 2022); CB Insights separately cites $54.21m raised in a corporate-minority round April 2022 — the two figures are not fully reconciled across sources, treat total_funding_mn as approximate.</t>
+        </is>
+      </c>
+      <c r="CQ16" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="CU16" t="inlineStr">
+        <is>
+          <t>Group revenue widely reported at approx. EUR 2.2bn for 2024; operating in 20 regulated markets as of 2026, still expanding (Ghana Feb 2026, Spain pending)</t>
+        </is>
+      </c>
+      <c r="CY16" t="n">
+        <v>3</v>
+      </c>
+      <c r="CZ16" t="n">
+        <v>4</v>
+      </c>
+      <c r="DC16" t="n">
+        <v>3</v>
+      </c>
+      <c r="DD16" t="n">
+        <v>67</v>
+      </c>
+      <c r="DE16" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="DH16" t="inlineStr">
+        <is>
+          <t>https://kaizengaming.com/news/kaizen-gaming-acquires-gameplai-to-accelerate-ai-driven-sports-trading-innovation/ ; https://sbcnews.co.uk/sportsbook/2026/02/10/kaizen-gaming-betano-ghana/ ; https://sbcnews.co.uk/europe/2026/07/27/kaizen-betano-spain/ ; https://legalclarity.org/who-owns-betano-kaizen-gaming-allwyn-and-founders/ ; https://kaizengaming.com/technology/ ; https://www.edgetier.com/case-study/how-kaizen-leverages-real-time-insights-to-proactively-manage-cx-and-responsible-gaming/</t>
+        </is>
+      </c>
+      <c r="DI16" t="inlineStr">
+        <is>
+          <t>Strong recent trade-press coverage (2026) on market expansion and the GameplAI acquisition; financial figures (revenue, funding) are private-company estimates from secondary sources and not confirmed by audited filings. || W1=3: Builds owned brand and proprietary tech, not overtly anti-affiliate | W2=3: GameplAI AI-trading acquisition is one relevant bet, not systemic | W3=2: FIFA/Tottenham sponsorships are brand deals, not funnel alliances | W4=3: Native app with AI personalization, AI trivia; single-vertical experiments | W5=2: Sponsorship-driven brand awareness; audience mostly rented, not owned | D1=4: Sportsbook, casino, live casino across 20 markets, strong content | D2=4: Proprietary in-house platform plus newly acquired GameplAI trading tech | D3=4: 20 regulated markets incl. MGA; Spain licence secured mid-2026 | D4=2: No confirmed owned MoR; payments likely run via PSP partners | D5=4: 20 regulated markets across Europe, LatAm, Africa; EUR 2.2bn revenue | D6=4: FIFA/Tottenham global sponsor; trusted top brand in core markets | AI1=3: Data science on external/partner stack (Databricks); no frontier models | AI2=0: No shipped autonomous or agentic betting assistant found | AI3=0: No MCP/A2A/UCP/ACP adoption evidence found in research | AI4=1: AI-powered app sections shipped, not a primary conversational assistant | AI5=4: Individual-level personalization; app reports 75%+ recommendation accuracy | AI6=3: GameplAI plus 3000-staff data infra; proprietary trading/behavioral data | AI7=2: Strategic AI partner/acquirer (Databricks, GameplAI); not an AI platform others build on | F1=3: Profitable private operator; no public signs of funding strain | F2=4: EUR 2.2bn 2024 group revenue; continued market expansion implies profitability | F3=None: Runway/cash position not publicly disclosed (private company) | F4=None: Leverage/debt levels not publicly disclosed | F5=3: Allwyn/OPAP strategic investor relationship provides a capital-access route</t>
+        </is>
+      </c>
+      <c r="DJ16" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="DK16" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="DL16" t="inlineStr">
+        <is>
+          <t>sonnet/company-researcher</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Trustly Group AB</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Stockholm, Sweden</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>2008</v>
+      </c>
+      <c r="D17" t="n">
+        <v>950</v>
+      </c>
+      <c r="F17" t="n">
+        <v>10000</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Payments &amp; fintech</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Open-banking 'Pay by Bank' payment initiation: instant account-to-account deposits and payouts for operators, monetized via per-transaction merchant fees; no card networks involved.</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>B2B2C — sells to gambling operators (Caesars Digital, Hard Rock Bet, FanDuel, DraftKings) who embed it at checkout for end players</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>Uses ML/AI for payment-timing prediction and fraud scoring; no evidence of building or fine-tuning foundation models</t>
+        </is>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AA17" t="inlineStr">
+        <is>
+          <t>L0</t>
+        </is>
+      </c>
+      <c r="AC17" t="inlineStr">
+        <is>
+          <t>Transaction and bank-linkage data across 650M+ consumers reachable via 12,000+ connected banks</t>
+        </is>
+      </c>
+      <c r="AF17" t="inlineStr">
+        <is>
+          <t>Caesars Digital, Hard Rock Bet, FanDuel, DraftKings (deposits/payouts), Nordic Capital (majority owner since 2018), SlimPay (acquired, closed May 2026)</t>
+        </is>
+      </c>
+      <c r="AH17" t="inlineStr">
+        <is>
+          <t>Authorised Payment Institution under PSD2 in Sweden (Finansinspektionen), passported across EU/EEA (30+ markets); FCA-authorised in UK; US operations for gaming payments</t>
+        </is>
+      </c>
+      <c r="AK17" t="inlineStr">
+        <is>
+          <t>Markets responsible-gaming features built on open-banking transaction data (e.g. affordability signals), not a public RG policy statement</t>
+        </is>
+      </c>
+      <c r="AM17" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AN17" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AO17" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AP17" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AQ17" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AR17" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AS17" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AT17" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AV17" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AX17" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AZ17" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="BB17" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="BD17" t="n">
+        <v>5</v>
+      </c>
+      <c r="BI17" t="n">
+        <v>1</v>
+      </c>
+      <c r="BJ17" t="n">
+        <v>2</v>
+      </c>
+      <c r="BK17" t="n">
+        <v>3</v>
+      </c>
+      <c r="BL17" t="n">
+        <v>3</v>
+      </c>
+      <c r="BM17" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO17" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP17" t="n">
+        <v>4</v>
+      </c>
+      <c r="BQ17" t="n">
+        <v>4</v>
+      </c>
+      <c r="BR17" t="n">
+        <v>4</v>
+      </c>
+      <c r="BS17" t="n">
+        <v>2</v>
+      </c>
+      <c r="BT17" t="n">
+        <v>2</v>
+      </c>
+      <c r="BU17" t="n">
+        <v>1</v>
+      </c>
+      <c r="BV17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX17" t="n">
+        <v>2</v>
+      </c>
+      <c r="BY17" t="n">
+        <v>3</v>
+      </c>
+      <c r="BZ17" t="n">
+        <v>1</v>
+      </c>
+      <c r="CA17" t="n">
+        <v>41</v>
+      </c>
+      <c r="CB17" t="n">
+        <v>41</v>
+      </c>
+      <c r="CC17" t="n">
+        <v>27</v>
+      </c>
+      <c r="CD17" t="n">
+        <v>34</v>
+      </c>
+      <c r="CE17" t="n">
+        <v>37</v>
+      </c>
+      <c r="CF17" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="CG17" t="inlineStr">
+        <is>
+          <t>Dormant</t>
+        </is>
+      </c>
+      <c r="CH17" t="inlineStr">
+        <is>
+          <t>No odds/content, no owned player audience, and not a full merchant-of-record — enables the wallet pillar for operators but shows no visible ambition to own the player relationship itself.</t>
+        </is>
+      </c>
+      <c r="CJ17" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="CK17" t="inlineStr">
+        <is>
+          <t>0-12m</t>
+        </is>
+      </c>
+      <c r="CL17" t="inlineStr">
+        <is>
+          <t>Makes deposits/payouts instant for whichever operator uses it, strengthening rather than bypassing the operator's own wallet — but Trustly concentrates the payments/wallet pillar, making it a likely partner or acquisition target for any future direct-to-player challenger.</t>
+        </is>
+      </c>
+      <c r="CN17" t="inlineStr">
+        <is>
+          <t>Legal entity Trustly Group AB, Stockholm; majority-owned by Nordic Capital since a 2018 take-private (~€700M). Distinct from 'Trust Payments' (UK-based rival, unrelated brand, avoid conflating in dedupe checks) and from crypto's 'Trust Wallet' (unrelated, surfaced in search noise). Currently exploring a ~$10B sale or IPO per October 2024 Bloomberg reporting; no confirmed outcome found as of this research (July 2026).</t>
+        </is>
+      </c>
+      <c r="CQ17" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="CU17" t="inlineStr">
+        <is>
+          <t>Q4 2025 revenue SEK 650M (+5% YoY constant currency), adj. EBITDA SEK 82.1M; ~$100B total payment volume processed in 2025, 120M+ users</t>
+        </is>
+      </c>
+      <c r="CY17" t="n">
+        <v>4</v>
+      </c>
+      <c r="CZ17" t="n">
+        <v>3</v>
+      </c>
+      <c r="DA17" t="n">
+        <v>4</v>
+      </c>
+      <c r="DC17" t="n">
+        <v>4</v>
+      </c>
+      <c r="DD17" t="n">
+        <v>75</v>
+      </c>
+      <c r="DE17" t="inlineStr">
+        <is>
+          <t>Stable</t>
+        </is>
+      </c>
+      <c r="DH17" t="inlineStr">
+        <is>
+          <t>https://www.trustly.com/press/trustly-surpasses-120-million-users-in-industry-leading-milestone-for-pay-by-bank ; https://www.trustly.com/press/trustly-launches-revolutionary-ai-powered-recurring-payments-to-boost-european-subscription-economy ; https://www.deucescracked.com/blog/trustly-slimpay-acquisition-igaming-payments-may-2026 ; https://www.bloomberg.com/news/articles/2024-10-11/nordic-capital-said-to-explore-options-for-payment-firm-trustly ; https://www.trustly.com/what-is-trustly</t>
+        </is>
+      </c>
+      <c r="DI17" t="inlineStr">
+        <is>
+          <t>Scale/product claims well-sourced from Trustly's own press releases; financial figures conflict between official Q4 press release (SEK 650M quarterly revenue) and a third-party estimate site (getlatka.com, ~$101M full-year) — the official figure is treated as more reliable, but exact FY2025 revenue is not independently confirmed, so confidence held at medium. Leverage (F4) genuinely unknown — private company. || W1=1: Invisible B2B payments rail; strengthens operators' wallets, no attack on model | W2=2: SlimPay deal expands recurring-payments infra, not player acquisition or AI | W3=3: Deep integrations with Caesars, FanDuel, DraftKings, Hard Rock — commercial | W4=3: Trustly ID (biometric login), Scan &amp; Pay, AI recurring payments shipped | W5=1: No owned discovery/intent audience — used only inside operator checkout | D1=0: No odds, markets or games content — pure payments infrastructure | D2=1: No PAM, bonusing or trading rail; payments-only infrastructure | D3=4: PSD2-passported across EU/EEA (30+ markets) plus UK FCA plus US ops | D4=4: Dominant Pay-by-Bank rail in EU iGaming, $100B+ volume, not full MoR | D5=4: 120M+ users, 30+ markets, 12,000 banks, ~$100B processed in 2025 | D6=2: Recognized checkout payment option, not a consumer destination brand | AI1=2: ML for payment-timing prediction/fraud; no evidence of own foundation models | AI2=1: AI predicts payment timing and fraud risk — assistive, not agentic | AI3=0: No evidence of MCP/A2A/UCP/ACP agent-commerce protocol adoption | AI4=0: No public customer-facing conversational assistant found | AI5=2: Post-SlimPay: predicts optimal payment timing per account, not offers | AI6=3: Transaction data across 650M+ linked consumers/12k banks is a real asset | AI7=1: Consumes AI/ML for internal fraud and payment-timing use only | F1=4: Nordic Capital-backed since 2018 (~€700M take-private); well-funded PE owner | F2=3: Positive adj. EBITDA (SEK 82.1M Q4 2025) but modest ~5% revenue growth | F3=4: PE-backed and EBITDA-positive; runway not a going-concern issue | F4=None: Private LBO-style capital structure; leverage terms not publicly disclosed | F5=4: Attempted Nasdaq Stockholm IPO at ~SEK75bn; now exploring ~$10B sale/IPO</t>
+        </is>
+      </c>
+      <c r="DJ17" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="DK17" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="DL17" t="inlineStr">
+        <is>
+          <t>sonnet/company-researcher</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
iGaming pilot complete: 25 companies populated, QA green
Final 8 (evoke, Kindred, Super Group, Underdog Fantasy, Pragmatic Play,
SoftSwiss, Paysafe, GeoComply) researched and ingested. Workbook now 25
companies; qa_check 10 passed / 0 warnings / 0 failures.

Cost confirmed after the revert: 222,975 tokens for 8 companies = 27.9k each,
matching batch 01's 27k and 2.4x better than the perAgent=1 canary's 68k.

Landscape shape so far: EPI 22-76, mean 45. Prediction-market/DFS challengers
top the table alongside Flutter (Underdog 73, Kalshi 69, Polymarket 64) while
incumbent operators and B2B suppliers cluster low - which is the frame working:
they are what is being disrupted, not the disruptors.

PROGRESS.md carries the measured cost and a scope note: the remaining ~105
companies are ~2.9M tokens, worth deciding before running the long tail.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/industries/igaming/igaming_landscape.xlsx
+++ b/industries/igaming/igaming_landscape.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DL20"/>
+  <dimension ref="A1:DL28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6897,6 +6897,2610 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>evoke plc</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>London, UK (Gibraltar-headquartered gaming operations)</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>1997</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Operator (B2C)</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Multi-brand licensed betting and gaming operator (William Hill, 888, Mr Green, 888poker); earns margin on sportsbook, casino and poker wagers, funded historically by heavy affiliate/paid-search acquisition spend.</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>B2C bettors/gamblers, primarily UK with select European and international markets</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="W21" t="inlineStr">
+        <is>
+          <t>Vendor/third-party AI tools used for app personalisation; no proprietary model development found</t>
+        </is>
+      </c>
+      <c r="Y21" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AA21" t="inlineStr">
+        <is>
+          <t>L0</t>
+        </is>
+      </c>
+      <c r="AC21" t="inlineStr">
+        <is>
+          <t>Decades of William Hill sportsbook pricing/trading data; not confirmed industry-defining</t>
+        </is>
+      </c>
+      <c r="AF21" t="inlineStr">
+        <is>
+          <t>Inspired Entertainment (extended long-term virtual sports retail partnership, 2025)</t>
+        </is>
+      </c>
+      <c r="AH21" t="inlineStr">
+        <is>
+          <t>UK Gambling Commission plus multiple EU/EEA jurisdictions (Gibraltar-based group); exited some non-core markets</t>
+        </is>
+      </c>
+      <c r="AI21" t="n">
+        <v>100</v>
+      </c>
+      <c r="AK21" t="inlineStr">
+        <is>
+          <t>History of large UK AML/responsible-gambling fines (888 entities, 2023); investing in updated player-protection tooling</t>
+        </is>
+      </c>
+      <c r="AL21" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AM21" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AN21" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AO21" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AP21" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AQ21" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AR21" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AS21" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AT21" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AV21" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AX21" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AZ21" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="BB21" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="BD21" t="n">
+        <v>4</v>
+      </c>
+      <c r="BI21" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ21" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK21" t="n">
+        <v>1</v>
+      </c>
+      <c r="BL21" t="n">
+        <v>2</v>
+      </c>
+      <c r="BM21" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN21" t="n">
+        <v>4</v>
+      </c>
+      <c r="BO21" t="n">
+        <v>4</v>
+      </c>
+      <c r="BP21" t="n">
+        <v>4</v>
+      </c>
+      <c r="BQ21" t="n">
+        <v>3</v>
+      </c>
+      <c r="BR21" t="n">
+        <v>3</v>
+      </c>
+      <c r="BS21" t="n">
+        <v>3</v>
+      </c>
+      <c r="BT21" t="n">
+        <v>2</v>
+      </c>
+      <c r="BU21" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV21" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW21" t="n">
+        <v>1</v>
+      </c>
+      <c r="BX21" t="n">
+        <v>3</v>
+      </c>
+      <c r="BY21" t="n">
+        <v>2</v>
+      </c>
+      <c r="BZ21" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA21" t="n">
+        <v>19</v>
+      </c>
+      <c r="CB21" t="n">
+        <v>73</v>
+      </c>
+      <c r="CC21" t="n">
+        <v>22</v>
+      </c>
+      <c r="CD21" t="n">
+        <v>48</v>
+      </c>
+      <c r="CE21" t="n">
+        <v>36</v>
+      </c>
+      <c r="CF21" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="CG21" t="inlineStr">
+        <is>
+          <t>Dormant</t>
+        </is>
+      </c>
+      <c r="CH21" t="inlineStr">
+        <is>
+          <t>No owned/direct acquisition strategy or agentic AI; still affiliate-dependent, debt-burdened and now weighing a sale of the Group.</t>
+        </is>
+      </c>
+      <c r="CJ21" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="CK21" t="inlineStr">
+        <is>
+          <t>0-12m</t>
+        </is>
+      </c>
+      <c r="CL21" t="inlineStr">
+        <is>
+          <t>Reinforces rather than disrupts the incumbent affiliate-buying model — explicitly cited in the brief's own framing as an 888/evoke example of players bought via Better Collective/Catena/Google.</t>
+        </is>
+      </c>
+      <c r="CN21" t="inlineStr">
+        <is>
+          <t>Formerly 888 Holdings plc; brands include William Hill, 888, Mr Green, 888poker, Mr Green. Explicitly named in the researcher brief's incumbent description as an example of the affiliate-buying operator model under threat, so scored within the low-willingness incumbent cluster alongside Betsson/Entain. Currently in a Board-announced strategic review including possible sale of the Group or units (2026) — treated as a financial-distress signal (survival_tier At-risk) rather than a willingness signal.</t>
+        </is>
+      </c>
+      <c r="CQ21" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="CU21" t="inlineStr">
+        <is>
+          <t>H1 2025 revenue €887.8m (+3% YoY); Q1 2026 trading described as starting 'positively', in line with own expectations</t>
+        </is>
+      </c>
+      <c r="CY21" t="n">
+        <v>2</v>
+      </c>
+      <c r="CZ21" t="n">
+        <v>2</v>
+      </c>
+      <c r="DA21" t="n">
+        <v>3</v>
+      </c>
+      <c r="DB21" t="n">
+        <v>1</v>
+      </c>
+      <c r="DC21" t="n">
+        <v>2</v>
+      </c>
+      <c r="DD21" t="n">
+        <v>40</v>
+      </c>
+      <c r="DE21" t="inlineStr">
+        <is>
+          <t>At-risk</t>
+        </is>
+      </c>
+      <c r="DH21" t="inlineStr">
+        <is>
+          <t>https://www.ajbell.co.uk/news/articles/brief-evoke-starts-2026-positively-confirms-2025-expectations ; https://www.yogonet.com/international/news/2025/10/06/115669-evoke-launches-upgraded-william-hill-vegas-app-website-in-the-uk ; https://kalkinemedia.com/uk/news/announcements/evoke-plc-evok-sets-12-august-2026-for-h1-interim-results-release-owner-of-william-hill-and-888-announces-key-investor-date</t>
+        </is>
+      </c>
+      <c r="DI21" t="inlineStr">
+        <is>
+          <t>Resolved to evoke plc (LSE: EVOK), formerly 888 Holdings plc, renamed 2023 after completing acquisition of William Hill International from Caesars (2022). Board announced in 2026 it is reviewing strategic options including a potential sale of the Group or business units, while confirming Q1 2026 trading in line with expectations. AI evidence limited to one confirmed shipped feature (AI-powered personalisation in the relaunched William Hill Vegas app, Oct 2025); no evidence found of agentic capability, commerce protocols, or a differentiated conversational assistant. || W1=0: Named in brief itself as buying players via affiliates/Google | W2=1: William Hill deal was scale consolidation, not player/AI/wallet bet | W3=1: Only Inspired virtual-sports retail deal found; no funnel alliances | W4=2: William Hill Vegas app relaunched with AI personalisation, Oct 2025 | W5=1: Audience largely rented via Better Collective/Catena/Google, per brief | D1=4: Full-vertical content: sportsbook, casino, live casino, poker | D2=4: Proprietary William Hill/888 trading and platform stack at scale | D3=4: Broad UK/EU licence portfolio; narrower than global majors | D4=3: Licensed operator; payments via PSP partners, owns player wallet | D5=3: Multi-market UK/Europe/select international, not global scale | D6=3: Storied William Hill brand trust dented by past AML/RG fines | AI1=2: Vendor AI powers app personalisation; no own model work found | AI2=0: No agentic assistant or autonomous transaction capability found | AI3=0: No MCP/A2A/UCP/ACP protocol adoption evidence found | AI4=1: Only generic support chat; no differentiated AI assistant | AI5=3: AI-powered personalisation live in William Hill Vegas app (2025) | AI6=2: Decades of William Hill pricing/trading data; not industry-defining moat | AI7=0: Pure consumer of third-party AI tools, no platform position | F1=2: Active strategic review incl. possible sale signals funding strain | F2=2: Revenue growing modestly but historically loss-making at net level | F3=3: Real operating revenue base; no imminent-collapse signal found | F4=1: High net debt from William Hill acquisition; leveraged balance sheet | F5=2: LSE-listed with public capital access, weakened by depressed valuation</t>
+        </is>
+      </c>
+      <c r="DJ21" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="DK21" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="DL21" t="inlineStr">
+        <is>
+          <t>sonnet/company-researcher</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>GeoComply Solutions</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Vancouver, Canada</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>2011</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>RegTech &amp; compliance</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Licenses a 'digital identity platform' (geolocation compliance, device intelligence, KYC, fraud detection) to regulated online-gambling operators and adjacent regulated industries on a SaaS/usage basis; near-mandatory infrastructure in US regulated sports-betting states.</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>B2B — geolocation, device-intelligence, KYC and fraud-detection infrastructure for regulated iGaming operators (DraftKings, FanDuel, MGM, Caesars, Hard Rock) plus streaming/media and fintech clients</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="W22" t="inlineStr">
+        <is>
+          <t>Trains proprietary ML models for geolocation/device/behavioral fraud detection at scale; no evidence of generative foundation-model development</t>
+        </is>
+      </c>
+      <c r="Y22" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AA22" t="inlineStr">
+        <is>
+          <t>L0</t>
+        </is>
+      </c>
+      <c r="AC22" t="inlineStr">
+        <is>
+          <t>200M+ device installs and 2B+ monthly incoming signals across iGaming, streaming and fintech — likely the largest cross-industry location/device fraud dataset in the sector</t>
+        </is>
+      </c>
+      <c r="AF22" t="inlineStr">
+        <is>
+          <t>Caesars Entertainment (multi-year renewal/expansion, June 2026); Hard Rock Digital/Hard Rock Bet (expanded, May 2026); Dabble (90%+ KYC pass-rate case study); also DraftKings, FanDuel, MGM, Amazon Prime Video, BBC, Akamai, Sightline as named customers</t>
+        </is>
+      </c>
+      <c r="AM22" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AN22" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AO22" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AP22" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AQ22" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AR22" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AS22" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AT22" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AV22" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AX22" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AZ22" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="BB22" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="BD22" t="n">
+        <v>5</v>
+      </c>
+      <c r="BI22" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ22" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK22" t="n">
+        <v>2</v>
+      </c>
+      <c r="BL22" t="n">
+        <v>1</v>
+      </c>
+      <c r="BM22" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN22" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO22" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP22" t="n">
+        <v>4</v>
+      </c>
+      <c r="BQ22" t="n">
+        <v>0</v>
+      </c>
+      <c r="BR22" t="n">
+        <v>4</v>
+      </c>
+      <c r="BS22" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT22" t="n">
+        <v>3</v>
+      </c>
+      <c r="BU22" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV22" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW22" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX22" t="n">
+        <v>1</v>
+      </c>
+      <c r="BY22" t="n">
+        <v>5</v>
+      </c>
+      <c r="BZ22" t="n">
+        <v>2</v>
+      </c>
+      <c r="CA22" t="n">
+        <v>17</v>
+      </c>
+      <c r="CB22" t="n">
+        <v>20</v>
+      </c>
+      <c r="CC22" t="n">
+        <v>31</v>
+      </c>
+      <c r="CD22" t="n">
+        <v>26</v>
+      </c>
+      <c r="CE22" t="n">
+        <v>22</v>
+      </c>
+      <c r="CF22" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="CG22" t="inlineStr">
+        <is>
+          <t>Dormant</t>
+        </is>
+      </c>
+      <c r="CH22" t="inlineStr">
+        <is>
+          <t>No content, wallet, or player-facing brand — a pure trust/compliance layer with zero ambition or shipped capability to own the player relationship.</t>
+        </is>
+      </c>
+      <c r="CJ22" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="CK22" t="inlineStr">
+        <is>
+          <t>3y+</t>
+        </is>
+      </c>
+      <c r="CL22" t="inlineStr">
+        <is>
+          <t>Near-mandatory compliance/fraud infrastructure inside almost every regulated US operator (DraftKings, FanDuel, MGM, Caesars, Hard Rock) — strengthens and legitimizes the incumbent licensed model rather than bypassing it, though its device/location data moat could become strategically valuable to any AI-driven challenger needing trust infrastructure.</t>
+        </is>
+      </c>
+      <c r="CN22" t="inlineStr">
+        <is>
+          <t>Legal entity GeoComply Solutions Inc. (HQ Vancouver, Canada, founded 2011). Headcount conflicts across sources (Tracxn: 370; getlatka 2025: 509) — left ftes null rather than pick one. Total funding not disclosed anywhere found (minority growth investment led by Blackstone Growth/Atairos in 2023, amount undisclosed, later investors undisclosed too) — left total_funding_mn null per the no-invented-numbers rule. No subsidiary/duplicate risk identified against other igaming batch entries. Scored as a new archetype for this batch: a RegTech/compliance infra provider with near-zero willingness to disrupt the operator model (like the B2B-supplier anchors) but an unusually large proprietary device/location data moat (AI6=5) that a future AI-driven challenger could plausibly need to acquire or partner with for trust infrastructure.</t>
+        </is>
+      </c>
+      <c r="CQ22" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="CU22" t="inlineStr">
+        <is>
+          <t>~$56M estimated 2025 revenue (third-party estimate, getlatka); 200+ million device installs and 2+ billion monthly incoming insights feeding its AI/ML fraud models</t>
+        </is>
+      </c>
+      <c r="CY22" t="n">
+        <v>4</v>
+      </c>
+      <c r="CZ22" t="n">
+        <v>3</v>
+      </c>
+      <c r="DA22" t="n">
+        <v>4</v>
+      </c>
+      <c r="DC22" t="n">
+        <v>4</v>
+      </c>
+      <c r="DD22" t="n">
+        <v>75</v>
+      </c>
+      <c r="DE22" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="DH22" t="inlineStr">
+        <is>
+          <t>https://sbcamericas.com/2026/05/13/geocomply-expands-deal-with-hard-rock/ ; https://www.geocomply.com/news/dabble-introduces-geocomplys-digital-identity-platform-achieving-90-kyc-pass-rates-and-gaining-deeper-fraud-visibility-through-device-and-location-intelligence/ ; https://getlatka.com/companies/geocomply.com ; https://www.blackstone.com/news/press/geocomply-announces-blackstone-growth-and-atairos-as-its-first-institutional-investors/</t>
+        </is>
+      </c>
+      <c r="DI22" t="inlineStr">
+        <is>
+          <t>Partnership/product claims sourced from GeoComply's own newsroom (Dabble case study) and SBC Americas trade coverage (Hard Rock expansion, May 2026; Caesars renewal referenced June 2026). Scale figures (200M+ device installs, 2B+ monthly insights, $56M 2025 revenue) come from getlatka's third-party company profile, not company-disclosed financials, so held at medium confidence. Funding history (Blackstone Growth + Atairos as 'first institutional investors', Jan 2023 press release) confirmed via Blackstone's own newsroom, but the investment amount was explicitly undisclosed in all sources found; later investors (Norwest, Arctos Partners, Elysian Park Ventures) appear in Tracxn's investor list without round sizes. || W1=0: Pure compliance/infra vendor; no ambition to own the player relationship | W2=1: PE growth capital raised for market expansion, not player-acquisition/AI/wallet bets | W3=2: Deep 2026 renewals with Caesars/Hard Rock; standard vendor deals, not funnel-reshaping | W4=1: Digital identity platform is a shipped, expanding B2B suite; no owned consumer surface | W5=0: Zero owned player audience; invisible background infra used by operators | D1=0: No odds, markets or games content — pure compliance/fraud infrastructure | D2=0: No PAM, wallet, trading or bonusing engine — not a betting platform | D3=4: Certified compliance/geolocation infra across virtually all regulated US igaming states | D4=0: No payments or MoR function; pure trust/compliance layer | D5=4: 200M+ device installs, 2B+ monthly insights; near-ubiquitous across regulated US states | D6=0: Invisible background infra; no player-facing brand or deposit relationship | AI1=3: Trains proprietary ML/fraud models (not frontier LLMs) at scale on 2B+ monthly signals | AI2=0: No shipped autonomous agent capability found | AI3=0: No MCP/A2A/UCP/ACP adoption evidence found | AI4=0: No customer-facing conversational assistant identified | AI5=1: Individual-level risk/trust scoring exists, but not offer/content personalisation | AI6=5: 200M+ device installs, 2B+ monthly insights — an industry-defining fraud/location data moat | AI7=2: Major operators depend on its platform for trust infra, but not a gen-AI ecosystem player | F1=4: PE-backed (Blackstone Growth, Atairos, Norwest, Arctos) since 2023 plus historically profitable bootstrapped growth | F2=3: Est. ~$56M 2025 revenue (third-party estimate); profitability not independently confirmed | F3=4: PE-backed, expanding key client relationships in 2026; no distress signals found | F4=None: Private minority-investment structure; leverage/debt terms not disclosed | F5=4: Backed by Blackstone Growth, Atairos, Norwest, Arctos, Elysian Park — strong institutional capital access</t>
+        </is>
+      </c>
+      <c r="DJ22" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="DK22" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="DL22" t="inlineStr">
+        <is>
+          <t>sonnet/company-researcher</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Kindred Group plc</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Malta (plus Gibraltar, London, Stockholm offices); parent FDJ United headquartered in Paris, France</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>1997</v>
+      </c>
+      <c r="D23" t="n">
+        <v>2348</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Operator (B2C)</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Multi-brand online sportsbook, casino, poker and bingo operator (Unibet, 32Red, Maria Casino, Vlad Cazino et al.); now a wholly-owned subsidiary of France's FDJ United after FDJ's tender offer completed October 2024 (~90.7% tendered, €2.45bn deal).</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>B2C bettors/casino players, primarily Western/Northern Europe (Sweden, UK, Belgium, Denmark, Italy) plus Australia</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="Y23" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AA23" t="inlineStr">
+        <is>
+          <t>L0</t>
+        </is>
+      </c>
+      <c r="AC23" t="inlineStr">
+        <is>
+          <t>25+ years of player betting/casino data across ~1.7m actives; not confirmed as AI-leveraged</t>
+        </is>
+      </c>
+      <c r="AH23" t="inlineStr">
+        <is>
+          <t>Australia, Belgium, Denmark, Estonia, France, Gibraltar, Guernsey, Italy, Malta, Sweden, UK, Romania (exited North America by Q2 2024)</t>
+        </is>
+      </c>
+      <c r="AI23" t="n">
+        <v>100</v>
+      </c>
+      <c r="AK23" t="inlineStr">
+        <is>
+          <t>Early mover on Betfilter self-exclusion ad-blocking tool (2018) and Swedish BankID identity verification (2016)</t>
+        </is>
+      </c>
+      <c r="AL23" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AM23" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AN23" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AO23" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AP23" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AQ23" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AR23" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AS23" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AT23" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AV23" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AX23" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AZ23" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="BB23" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="BD23" t="n">
+        <v>4</v>
+      </c>
+      <c r="BI23" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ23" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK23" t="n">
+        <v>1</v>
+      </c>
+      <c r="BL23" t="n">
+        <v>1</v>
+      </c>
+      <c r="BM23" t="n">
+        <v>2</v>
+      </c>
+      <c r="BN23" t="n">
+        <v>4</v>
+      </c>
+      <c r="BO23" t="n">
+        <v>4</v>
+      </c>
+      <c r="BP23" t="n">
+        <v>4</v>
+      </c>
+      <c r="BQ23" t="n">
+        <v>3</v>
+      </c>
+      <c r="BR23" t="n">
+        <v>3</v>
+      </c>
+      <c r="BS23" t="n">
+        <v>3</v>
+      </c>
+      <c r="BT23" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU23" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV23" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW23" t="n">
+        <v>1</v>
+      </c>
+      <c r="BX23" t="n">
+        <v>1</v>
+      </c>
+      <c r="BY23" t="n">
+        <v>2</v>
+      </c>
+      <c r="BZ23" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA23" t="n">
+        <v>12</v>
+      </c>
+      <c r="CB23" t="n">
+        <v>73</v>
+      </c>
+      <c r="CC23" t="n">
+        <v>10</v>
+      </c>
+      <c r="CD23" t="n">
+        <v>42</v>
+      </c>
+      <c r="CE23" t="n">
+        <v>30</v>
+      </c>
+      <c r="CF23" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="CG23" t="inlineStr">
+        <is>
+          <t>Dormant</t>
+        </is>
+      </c>
+      <c r="CH23" t="inlineStr">
+        <is>
+          <t>No independent strategic agency post-acquisition; no confirmed AI, agentic, or direct-acquisition initiatives found.</t>
+        </is>
+      </c>
+      <c r="CJ23" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="CK23" t="inlineStr">
+        <is>
+          <t>0-12m</t>
+        </is>
+      </c>
+      <c r="CL23" t="inlineStr">
+        <is>
+          <t>Now absorbed into FDJ United's incumbent multi-brand affiliate-acquisition model as a subsidiary under active strategic/divestment review, rather than acting as an independent disruptor.</t>
+        </is>
+      </c>
+      <c r="CN23" t="inlineStr">
+        <is>
+          <t>Kindred Group plc was fully absorbed into FDJ United (La Française des Jeux) via a tender offer completed 3 Oct 2024; it now operates as a subsidiary, not an independent strategic actor. Flagship brand Unibet; also owns 32Red, Maria Casino, Vlad Cazino, iGame and others. Employee count (2,348) and Q3 2024 revenue figures are pre/near-acquisition and may not reflect post-integration reality. Scored within the low-willingness incumbent operator cluster (below Betsson) given the added signal of the parent's 2026 divestment review; AI dimension specifically has thin evidence and should be revisited with a dedicated Unibet-AI search before being treated as decision-critical.</t>
+        </is>
+      </c>
+      <c r="CQ23" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="CU23" t="inlineStr">
+        <is>
+          <t>Q3 2024 (pre-full integration): £294.5m quarterly revenue, 1.70m active customers</t>
+        </is>
+      </c>
+      <c r="CY23" t="n">
+        <v>3</v>
+      </c>
+      <c r="CZ23" t="n">
+        <v>2</v>
+      </c>
+      <c r="DA23" t="n">
+        <v>3</v>
+      </c>
+      <c r="DB23" t="n">
+        <v>2</v>
+      </c>
+      <c r="DC23" t="n">
+        <v>4</v>
+      </c>
+      <c r="DD23" t="n">
+        <v>56</v>
+      </c>
+      <c r="DE23" t="inlineStr">
+        <is>
+          <t>At-risk</t>
+        </is>
+      </c>
+      <c r="DH23" t="inlineStr">
+        <is>
+          <t>https://www.fdjunited.com/presse/fdjs-tender-offer-for-kindred-succeeds-creating-a-european-gaming-champion/ ; https://igamingbusiness.com/strategy/ma/fdj-completes-acquisition-kindred-group/ ; https://next.io/news/investment/fdj-review-online-gaming-business-after-kindred-acquisition/ ; https://en.wikipedia.org/wiki/Kindred_Group</t>
+        </is>
+      </c>
+      <c r="DI23" t="inlineStr">
+        <is>
+          <t>FDJ's tender offer for Kindred succeeded 3 Oct 2024 (90.66% of shares tendered), completing a EUR2.45bn acquisition and creating 'FDJ United'. FDJ financed the deal partly via a EUR1.5bn inaugural bond issue. As of H1 2026 reporting, FDJ United is conducting a market review of the online-gaming business signalling possible divestment/market exits, which is the main recent strategic signal available. No AI-specific evidence for Kindred/Unibet surfaced in the searches run (which were acquisition- and entity-focused, not AI-focused) — AI scores here are consequently thin and sit below the batch-01 AI floor (Evolution 16%); flagged as low-confidence and a candidate for a dedicated follow-up search if this company becomes decision-critical. || W1=0: Absorbed into FDJ United; no independent direct-player strategy found | W2=0: No AI/prediction/wallet M&amp;A; only consolidation into FDJ United | W3=1: Historical sports sponsorship deals; no funnel-repositioning alliances found | W4=1: Standard Unibet app only; no AI assistant or prediction surface found | W5=2: Some Unibet brand loyalty, but mostly affiliate/SEO-driven traffic | D1=4: Multi-vertical: sportsbook, casino, live casino, poker/bingo brands | D2=4: Proprietary Unibet trading/pricing platform at scale historically | D3=4: Broad European licence portfolio across 12 jurisdictions | D4=3: Licensed operator; payments via PSP partners, owns player wallet | D5=3: 1.7m actives, multi-market Europe/Australia, not global scale | D6=3: Unibet respected in Nordic/UK niche, not globally top-of-mind | AI1=0: No evidence found of foundation-model use or development | AI2=0: No shipped agentic capability found | AI3=0: No MCP/A2A/UCP/ACP adoption evidence found | AI4=1: Likely only generic support chat; no differentiated assistant found | AI5=1: No confirmed AI personalisation feature found for Unibet/Kindred | AI6=2: 25+ years of player data across 1.7m actives; unconfirmed AI use | AI7=0: No evidence of platform position in gen-AI ecosystem | F1=3: Backed by well-capitalized parent FDJ United post-acquisition | F2=2: Historically profitable, but unit now under strategic review | F3=3: Parent-backed; no near-term runway concern identified | F4=2: FDJ took on significant debt (EUR1.5bn bond) to fund deal | F5=4: Parent FDJ United is a large listed group with bond-market access</t>
+        </is>
+      </c>
+      <c r="DJ23" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="DK23" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="DL23" t="inlineStr">
+        <is>
+          <t>sonnet/company-researcher</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Paysafe Limited</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>London, UK (incorporated in Bermuda; NYSE: PSFE)</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>1996</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Payments &amp; fintech</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Merchant acquiring, payment gateway and processing (~$150B annual volume) for high-risk sectors incl. iGaming, plus owned Skrill and Neteller e-wallets giving players a direct funding/payout account; publicly traded on NYSE.</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>B2B2C — high-risk merchant acquiring/payment processing for iGaming operators, plus owned Skrill and Neteller e-wallets used directly by millions of players</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="W24" t="inlineStr">
+        <is>
+          <t>Integrates with third-party LLM platforms (OpenAI ChatGPT, Anthropic Claude, Google Gemini) for agentic commerce; no evidence of building own foundation models</t>
+        </is>
+      </c>
+      <c r="Y24" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AA24" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="AC24" t="inlineStr">
+        <is>
+          <t>Two decades of high-risk gambling payment/fraud data across $150B annual volume and 7.9M wallet users</t>
+        </is>
+      </c>
+      <c r="AD24" t="inlineStr">
+        <is>
+          <t>ChatGPT, Claude, Gemini agentic-commerce payment integration (2026)</t>
+        </is>
+      </c>
+      <c r="AF24" t="inlineStr">
+        <is>
+          <t>Agentic-commerce payment integrations with ChatGPT, Claude and Gemini (announced 2026); owns Skrill and Neteller e-wallet brands</t>
+        </is>
+      </c>
+      <c r="AH24" t="inlineStr">
+        <is>
+          <t>FCA e-money institution (Paysafe Financial Services Limited, FRN 900015), UK; additional EU/international payment licences not itemized in sources reviewed this session</t>
+        </is>
+      </c>
+      <c r="AL24" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AM24" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AN24" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AO24" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AP24" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AQ24" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AR24" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AS24" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AT24" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AV24" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AX24" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AZ24" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="BB24" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="BD24" t="n">
+        <v>5</v>
+      </c>
+      <c r="BI24" t="n">
+        <v>3</v>
+      </c>
+      <c r="BJ24" t="n">
+        <v>2</v>
+      </c>
+      <c r="BK24" t="n">
+        <v>3</v>
+      </c>
+      <c r="BL24" t="n">
+        <v>3</v>
+      </c>
+      <c r="BM24" t="n">
+        <v>3</v>
+      </c>
+      <c r="BN24" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO24" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP24" t="n">
+        <v>4</v>
+      </c>
+      <c r="BQ24" t="n">
+        <v>5</v>
+      </c>
+      <c r="BR24" t="n">
+        <v>4</v>
+      </c>
+      <c r="BS24" t="n">
+        <v>4</v>
+      </c>
+      <c r="BT24" t="n">
+        <v>2</v>
+      </c>
+      <c r="BU24" t="n">
+        <v>2</v>
+      </c>
+      <c r="BV24" t="n">
+        <v>1</v>
+      </c>
+      <c r="BW24" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX24" t="n">
+        <v>2</v>
+      </c>
+      <c r="BY24" t="n">
+        <v>4</v>
+      </c>
+      <c r="BZ24" t="n">
+        <v>3</v>
+      </c>
+      <c r="CA24" t="n">
+        <v>55</v>
+      </c>
+      <c r="CB24" t="n">
+        <v>48</v>
+      </c>
+      <c r="CC24" t="n">
+        <v>40</v>
+      </c>
+      <c r="CD24" t="n">
+        <v>44</v>
+      </c>
+      <c r="CE24" t="n">
+        <v>48</v>
+      </c>
+      <c r="CF24" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="CG24" t="inlineStr">
+        <is>
+          <t>Dormant</t>
+        </is>
+      </c>
+      <c r="CH24" t="inlineStr">
+        <is>
+          <t>No odds/games content and no owned betting surface — wallet and emerging agentic-payment rails only; would need a product/content play to complete the three-pillar bypass.</t>
+        </is>
+      </c>
+      <c r="CJ24" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="CK24" t="inlineStr">
+        <is>
+          <t>0-12m</t>
+        </is>
+      </c>
+      <c r="CL24" t="inlineStr">
+        <is>
+          <t>Owns two of iGaming's most-used player wallets (Skrill, Neteller) and is now building agent-initiated payment rails across ChatGPT/Claude/Gemini — positioned to become the wallet pillar for any AI-driven bypass of operator acquisition, not just a passive payments vendor.</t>
+        </is>
+      </c>
+      <c r="CN24" t="inlineStr">
+        <is>
+          <t>Legal entity Paysafe Limited (Bermuda-incorporated, NYSE: PSFE, HQ operations London); owns Skrill Limited, Neteller (Paysafe (Isle of Man) Limited) and the Paysafecard prepaid-voucher brand as subsidiaries of the same group — not separate companies, avoid double-counting if any of those brands surface elsewhere in the batch. Company has a leveraged-buyout history (Blackstone/CVC took it private in 2017; relisted via SPAC merger with Foley Trasimene Acquisition Corp II in 2021) that plausibly still affects its balance sheet (F4), but current leverage figures were not independently verified within this session's research budget.</t>
+        </is>
+      </c>
+      <c r="CQ24" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="CU24" t="inlineStr">
+        <is>
+          <t>FY2025 revenue $1.70B (flat YoY); Q1 2026 revenue $442.7M (+10% YoY); FY2026 guidance $1.79-1.83B; iGaming revenue +28% YoY and wallet revenue +15% to $216.3M in Q1 2026</t>
+        </is>
+      </c>
+      <c r="CY24" t="n">
+        <v>4</v>
+      </c>
+      <c r="CZ24" t="n">
+        <v>2</v>
+      </c>
+      <c r="DA24" t="n">
+        <v>3</v>
+      </c>
+      <c r="DC24" t="n">
+        <v>4</v>
+      </c>
+      <c r="DD24" t="n">
+        <v>65</v>
+      </c>
+      <c r="DE24" t="inlineStr">
+        <is>
+          <t>Stable</t>
+        </is>
+      </c>
+      <c r="DH24" t="inlineStr">
+        <is>
+          <t>https://www.pymnts.com/earnings/2026/paysafe-targets-agentic-commerce-as-digital-wallet-users-jump-9percent/ ; https://www.paysafe.com/us-en/paysafegroup/news/detail/paysafe-reports-first-quarter-2026-results/ ; https://thefinrate.com/paysafe-review-2026-high-risk-merchant-accounts-fees-approval-rates/ ; https://www.stocktitan.net/sec-filings/PSFE/6-k-paysafe-ltd-current-report-foreign-issuer-703dcd241eb0.html</t>
+        </is>
+      </c>
+      <c r="DI24" t="inlineStr">
+        <is>
+          <t>PYMNTS earnings coverage (Q1 2026) fetched directly: CEO Bruce Lowthers quoted that 'with one integration, Paysafe can enable merchants to offer AI powered commerce across ChatGPT, Claude, and Gemini' — real and dated, but framed as a capability being rolled out, not confirmed at full production scale, and no specific agent-commerce protocol (MCP/ACP/UCP/A2A) was named in the coverage reviewed. Financials cross-checked against Paysafe's own Q1 2026 results release and a StockTitan SEC 6-K filing note ('posts 2025 loss, guides to stronger 2026'). High-risk/MoR positioning and $150B volume figure sourced from a third-party merchant-services review site (thefinrate.com), so held at medium confidence pending primary-source confirmation. || W1=3: Publicly building agentic-commerce payment rails (ChatGPT/Claude/Gemini), not just legacy processing | W2=2: Investing in agentic-commerce infra; no player-acquisition/prediction-market M&amp;A found | W3=3: Live integrations with ChatGPT, Claude and Gemini for AI-initiated commerce | W4=3: Skrill/Neteller are live, owned consumer wallets with millions of iGaming users | W5=3: 7.9M active wallet users skew heavily toward iGaming; real owned audience | D1=0: No odds, markets or games content — pure payments infrastructure | D2=1: No PAM/trading/bonusing rail; wallet infrastructure only | D3=4: FCA e-money institution; decades of high-risk/iGaming compliance expertise | D4=5: Direct high-risk gambling merchant acquirer, $150B processing volume, owns Skrill/Neteller | D5=4: $150B annual volume, 7.9M wallet users across UK/EU/LatAm and beyond | D6=4: Skrill/Neteller are decades-old, widely trusted iGaming wallet brands players deposit into directly | AI1=2: Integrates with external LLM platforms (ChatGPT, Claude, Gemini), not own models | AI2=2: Agent-checkout capability announced across 3 AI platforms; live-at-scale status unclear | AI3=1: Multi-platform AI-checkout capability announced; specific protocol (MCP/ACP) unconfirmed | AI4=0: No dedicated own customer-facing conversational assistant identified | AI5=2: AI-driven customer acquisition campaigns in Europe; personalisation depth unclear | AI6=4: Deep high-risk gambling transaction data across $150B volume and 7.9M wallet users | AI7=3: Strategic payment-rail partner across ChatGPT, Claude and Gemini agentic commerce | F1=4: Public company (NYSE: PSFE) with $1.7B+ revenue base; adequate funding | F2=2: FY2025 net loss reported despite $1.7B revenue; 2026 guidance calls for growth | F3=3: Public, ongoing operations; no going-concern flags found this session | F4=None: Historically leveraged (post-2017 take-private); current debt levels not verified this session | F5=4: NYSE-listed public company; access to public equity/debt capital markets</t>
+        </is>
+      </c>
+      <c r="DJ24" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="DK24" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="DL24" t="inlineStr">
+        <is>
+          <t>sonnet/company-researcher</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Pragmatic Play</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Malta (operating hub); ultimate owner Veridian (Gibraltar) Limited</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>2015</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>B2B supplier &amp; platform</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Licenses proprietary slots, live-casino tables and bingo content to operators for revenue-share/fees; wound down sportsbook, virtual sports and bingo in June 2026 to refocus purely on slots and live casino.</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>B2B — licenses slots/live-casino content to 8,000+ regulated operators worldwide; no direct consumer wallet or brand</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="W25" t="inlineStr">
+        <is>
+          <t>No evidence of building, fine-tuning, or disclosed use of foundation models</t>
+        </is>
+      </c>
+      <c r="Y25" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AA25" t="inlineStr">
+        <is>
+          <t>L0</t>
+        </is>
+      </c>
+      <c r="AC25" t="inlineStr">
+        <is>
+          <t>Broad gameplay/telemetry data across 8,000+ operators and 150+ markets; not confirmed to power any visible AI product</t>
+        </is>
+      </c>
+      <c r="AF25" t="inlineStr">
+        <is>
+          <t>8,000+ operator integrations; ARRISE (affiliated services/dev partner, Gibraltar, ~6,000 staff); GR8 Tech (aggregator distribution)</t>
+        </is>
+      </c>
+      <c r="AH25" t="inlineStr">
+        <is>
+          <t>40+ licensed jurisdictions incl. MGA, UKGC, Gibraltar Gambling Commissioner; content live in 150+ markets</t>
+        </is>
+      </c>
+      <c r="AM25" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AN25" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AO25" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AP25" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AQ25" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AR25" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AS25" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AT25" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AV25" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AX25" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AZ25" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="BB25" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="BD25" t="n">
+        <v>2</v>
+      </c>
+      <c r="BI25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK25" t="n">
+        <v>1</v>
+      </c>
+      <c r="BL25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN25" t="n">
+        <v>5</v>
+      </c>
+      <c r="BO25" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP25" t="n">
+        <v>5</v>
+      </c>
+      <c r="BQ25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BR25" t="n">
+        <v>5</v>
+      </c>
+      <c r="BS25" t="n">
+        <v>3</v>
+      </c>
+      <c r="BT25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX25" t="n">
+        <v>1</v>
+      </c>
+      <c r="BY25" t="n">
+        <v>2</v>
+      </c>
+      <c r="BZ25" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA25" t="n">
+        <v>4</v>
+      </c>
+      <c r="CB25" t="n">
+        <v>61</v>
+      </c>
+      <c r="CC25" t="n">
+        <v>8</v>
+      </c>
+      <c r="CD25" t="n">
+        <v>34</v>
+      </c>
+      <c r="CE25" t="n">
+        <v>22</v>
+      </c>
+      <c r="CF25" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="CG25" t="inlineStr">
+        <is>
+          <t>Dormant</t>
+        </is>
+      </c>
+      <c r="CH25" t="inlineStr">
+        <is>
+          <t>No player-facing platform, wallet, payments or owned audience — everything reaches players only through operator brands.</t>
+        </is>
+      </c>
+      <c r="CJ25" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="CK25" t="inlineStr">
+        <is>
+          <t>3y+</t>
+        </is>
+      </c>
+      <c r="CL25" t="inlineStr">
+        <is>
+          <t>Supplies must-have slots/live-casino content that keeps players inside operator brands — reinforces the incumbent acquisition funnel rather than bypassing it.</t>
+        </is>
+      </c>
+      <c r="CN25" t="inlineStr">
+        <is>
+          <t>Resolved to Pragmatic Play as the content-licensing entity (parent: Veridian (Gibraltar) Limited); kept distinct from ARRISE (affiliated services/dev company, ~6,000 staff, separate entity) to avoid conflating headcount/revenue. Per July 2026 reporting, Pragmatic Play wound down sportsbook, virtual sports and bingo in June 2026 to refocus on slots and live casino — verticals scored accordingly (bingo dropped despite historical offering). Scored consistently with the Evolution AB anchor (Dormant, invisible-to-player B2B content supplier, near-zero willingness) but with slightly higher D1/D5 given Pragmatic's broader slots+live-casino footprint across more markets and operators.</t>
+        </is>
+      </c>
+      <c r="CQ25" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="CU25" t="inlineStr">
+        <is>
+          <t>~$750M estimated annual revenue (Aug 2025 estimate, unverified/conflicting with other directory figures)</t>
+        </is>
+      </c>
+      <c r="CY25" t="n">
+        <v>4</v>
+      </c>
+      <c r="CZ25" t="n">
+        <v>3</v>
+      </c>
+      <c r="DA25" t="n">
+        <v>4</v>
+      </c>
+      <c r="DC25" t="n">
+        <v>2</v>
+      </c>
+      <c r="DD25" t="n">
+        <v>65</v>
+      </c>
+      <c r="DE25" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="DH25" t="inlineStr">
+        <is>
+          <t>https://todaynews.co.uk/2026/07/14/how-is-pragmatic-play-structured-veridian-arrise-and-julian-jarvis/ ; https://igamingexpress.com/who-owns-pragmatic-play/ ; https://sigma.world/news/all-about-pragmatic-play/ ; https://punchng.com/pragmatic-play-company-history-from-startup-to-500-slots-and-a-global-live-casino-in-under-10-years/</t>
+        </is>
+      </c>
+      <c r="DI25" t="inlineStr">
+        <is>
+          <t>Ownership resolved via Veridian (Gibraltar) Limited / CEO Julian Jarvis reporting (todaynews.co.uk, iGaming Express, July 2026). Scale figures (40+ licences, 150+ markets, 8,000+ operators, 500+ titles) corroborated across SiGMA and Punch Newspapers company-history pieces. Revenue is genuinely uncertain — one estimate puts it near $750M (Aug 2025), while a company-directory site shows an implausible $25.8M figure for 2026; treated the former as directionally more credible but flagged unverified. No AI-specific product, MCP/A2A/UCP/ACP, or customer-facing assistant evidence surfaced in searches focused on ARRISE/Pragmatic Play AI activity. || W1=0: No public strategy to own player relationship; pure B2B content supplier | W2=0: No M&amp;A toward player-acquisition, AI, prediction or wallet assets found | W3=1: Standard operator/aggregator supply deals, not funnel-reshaping alliances | W4=0: No owned app, wallet or AI assistant shipped to players | W5=0: Zero owned audience; retrenched further by exiting sportsbook/virtuals in 2026 | D1=5: Dominant slots/live-casino content; must-have for those verticals, no sportsbook now | D2=1: No PAM/wallet/trading rail; API-delivered content platform only | D3=5: 40+ jurisdictions incl. MGA/UKGC; broad tier-1 compliance machine | D4=0: No payments or MoR function; pure content licensor | D5=5: Live with 8,000+ operators across 150+ regulated jurisdictions | D6=3: Recognized, quality-associated content brand among players; not a deposit destination | AI1=0: No public evidence of foundation-model use or development | AI2=0: No shipped agentic capability found | AI3=0: No MCP/A2A/UCP/ACP adoption evidence found | AI4=0: No customer-facing conversational assistant identified | AI5=1: Likely basic in-game recommendation only; no disclosed AI personalization engine | AI6=2: Massive gameplay telemetry across 8,000+ operators, but no confirmed AI product use | AI7=0: No evidence of others building on Pragmatic Play AI; pure content vendor | F1=4: Self-funded via revenue at scale since 2015; no external funding rounds found | F2=3: Est. ~$750M revenue (unverified); profitability not publicly disclosed | F3=4: Decade+ of stable, scaled operations; no distress signals found | F4=None: Private company; leverage/debt terms not disclosed | F5=2: Privately held, no public listing; capital access via owner (Veridian) not disclosed</t>
+        </is>
+      </c>
+      <c r="DJ25" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="DK25" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="DL25" t="inlineStr">
+        <is>
+          <t>sonnet/company-researcher</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>SoftSwiss</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>St. Julian's, Malta</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>2009</v>
+      </c>
+      <c r="D26" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>B2B supplier &amp; platform</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Licenses a full-stack iGaming platform (PAM, game aggregator with 30,000+ games, sportsbook, jackpot aggregator, crypto/fiat payments, and a new 2026 Prediction Markets product) to operators for fees/revenue share; bootstrapped, no external funding.</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>B2B — powers 1,500+ regulated iGaming/casino operator brands with platform, game-aggregation, sportsbook and payments infrastructure</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="W26" t="inlineStr">
+        <is>
+          <t>Proprietary ML (anti-fraud, behavior-tracking) layered on external AI tooling; no evidence of training foundation models</t>
+        </is>
+      </c>
+      <c r="Y26" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AA26" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="AC26" t="inlineStr">
+        <is>
+          <t>Player behavioral/transaction data across 1,500+ operator brands plus native crypto-payment rails</t>
+        </is>
+      </c>
+      <c r="AF26" t="inlineStr">
+        <is>
+          <t>TrueLabel (sportsbook integration, Feb 2026); 1,500+ iGaming operator brands; new AI-focused C-level executive hire (Jan 2026)</t>
+        </is>
+      </c>
+      <c r="AH26" t="inlineStr">
+        <is>
+          <t>24+ jurisdictions incl. Malta (MGA), Curacao, UK (UKGC), Sweden, Greece, Romania, Serbia, Brazil (SPA), Ontario (Canada), West Virginia (US), South Africa, Ghana</t>
+        </is>
+      </c>
+      <c r="AK26" t="inlineStr">
+        <is>
+          <t>Markets AI-driven behavior-tracking tools for responsible-gambling signals to operator clients</t>
+        </is>
+      </c>
+      <c r="AL26" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AM26" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AN26" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AO26" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AP26" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AQ26" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AR26" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AS26" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AT26" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AV26" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AX26" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AZ26" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="BB26" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="BD26" t="n">
+        <v>4</v>
+      </c>
+      <c r="BI26" t="n">
+        <v>1</v>
+      </c>
+      <c r="BJ26" t="n">
+        <v>3</v>
+      </c>
+      <c r="BK26" t="n">
+        <v>2</v>
+      </c>
+      <c r="BL26" t="n">
+        <v>1</v>
+      </c>
+      <c r="BM26" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN26" t="n">
+        <v>4</v>
+      </c>
+      <c r="BO26" t="n">
+        <v>5</v>
+      </c>
+      <c r="BP26" t="n">
+        <v>4</v>
+      </c>
+      <c r="BQ26" t="n">
+        <v>3</v>
+      </c>
+      <c r="BR26" t="n">
+        <v>4</v>
+      </c>
+      <c r="BS26" t="n">
+        <v>1</v>
+      </c>
+      <c r="BT26" t="n">
+        <v>2</v>
+      </c>
+      <c r="BU26" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV26" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW26" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX26" t="n">
+        <v>3</v>
+      </c>
+      <c r="BY26" t="n">
+        <v>3</v>
+      </c>
+      <c r="BZ26" t="n">
+        <v>3</v>
+      </c>
+      <c r="CA26" t="n">
+        <v>32</v>
+      </c>
+      <c r="CB26" t="n">
+        <v>76</v>
+      </c>
+      <c r="CC26" t="n">
+        <v>26</v>
+      </c>
+      <c r="CD26" t="n">
+        <v>51</v>
+      </c>
+      <c r="CE26" t="n">
+        <v>43</v>
+      </c>
+      <c r="CF26" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="CG26" t="inlineStr">
+        <is>
+          <t>Dormant</t>
+        </is>
+      </c>
+      <c r="CH26" t="inlineStr">
+        <is>
+          <t>No owned consumer brand or audience — despite the broadest B2B stack in the batch, it still has zero direct player relationship.</t>
+        </is>
+      </c>
+      <c r="CJ26" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="CK26" t="inlineStr">
+        <is>
+          <t>1-3y</t>
+        </is>
+      </c>
+      <c r="CL26" t="inlineStr">
+        <is>
+          <t>Powers the operator stack (platform, content, payments, now prediction markets) more deeply than most rivals, but still sells to operators rather than bypassing them — a rail beneath the incumbent, not yet a direct competitor.</t>
+        </is>
+      </c>
+      <c r="CN26" t="inlineStr">
+        <is>
+          <t>Legal entity SOFTSWISS (HQ Malta), founded 2009 by Ivan Montik and Dzmitry Yaikau, explicitly unfunded/bootstrapped. Distinct from BitStarz (operated by Dama N.V.), a crypto casino brand historically associated with SoftSwiss's founding team but now a separate operator entity — do not conflate if BitStarz appears elsewhere in the batch. Scored above the Kambi anchor (Dormant, B2B trading supplier) on willingness given SoftSwiss's explicit 2026 AI-vision push and new Prediction Markets product line, but kept low overall since it remains a B2B enabler with zero owned player audience or consumer brand.</t>
+        </is>
+      </c>
+      <c r="CQ26" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="CU26" t="inlineStr">
+        <is>
+          <t>~$420M estimated 2026 revenue (Tracxn estimate, unverified); 2,000+ employees across 30+ countries; 1,500+ operator brands served</t>
+        </is>
+      </c>
+      <c r="CY26" t="n">
+        <v>4</v>
+      </c>
+      <c r="CZ26" t="n">
+        <v>3</v>
+      </c>
+      <c r="DA26" t="n">
+        <v>4</v>
+      </c>
+      <c r="DC26" t="n">
+        <v>2</v>
+      </c>
+      <c r="DD26" t="n">
+        <v>65</v>
+      </c>
+      <c r="DE26" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="DH26" t="inlineStr">
+        <is>
+          <t>https://www.softswiss.com/news/softswiss-strategic-vision-2026/ ; https://sbcnews.co.uk/europe/2026/01/26/softswiss-ai-c-level-hire/ ; https://www.softswiss.com/prediction-markets-software/ ; https://techround.co.uk/tech/ivan-montik-founder-at-softswiss-on-staying-ahead-in-one-of-techs-fastest-moving-industries/</t>
+        </is>
+      </c>
+      <c r="DI26" t="inlineStr">
+        <is>
+          <t>SOFTSWISS's own 2026 strategic-vision post confirms a deliberate AI-driven-workflow push and a new Prediction Markets product (standalone widget or sportsbook-integrated, 2-3 week operator onboarding). SBC News (Jan 2026) confirms a new C-level AI-focused hire. Licensing/jurisdiction breadth and crypto-native payments (50+ currencies) corroborated across platform-comparison sites (tech-insider.org, bestwhitelabelcasinos.com). Revenue (~$420M) and headcount (2,000+) are third-party (Tracxn) estimates, not company-disclosed, so held at medium confidence. No MCP/A2A/UCP/ACP, agentic, or customer-facing-assistant evidence found. || W1=1: B2B enabler; no direct-to-player ambition despite new product categories | W2=3: Launched Prediction Markets product + hired AI-focused exec in 2026 | W3=2: TrueLabel/sportsbook integrations, 1,500+ operator deals; standard B2B supply | W4=1: New B2B products (prediction markets, sportsbook) shipped; no owned consumer surface | W5=0: No owned audience; purely B2B, zero direct player reach | D1=4: Aggregates 30,000+ games plus sportsbook and prediction markets; licensed-in, not own IP | D2=5: Core strength: proven owned PAM/casino/sportsbook platform used by 1,500+ brands | D3=4: 24+ regulated jurisdictions incl. MGA, UKGC, Brazil SPA, Ontario | D4=3: Built-in crypto/fiat payments infra (50+ cryptocurrencies), not full owned MoR | D5=4: 1,500+ operator brands live across 24+ jurisdictions; global platform footprint | D6=1: Backend platform brand, essentially invisible to end players | AI1=2: ML anti-fraud/behavior tracking built on external AI tooling, not frontier models | AI2=0: No shipped autonomous agent capability found | AI3=0: No MCP/A2A/UCP/ACP adoption evidence found | AI4=0: No customer-facing conversational assistant identified | AI5=3: ML behavior-tracking drives per-player retention/RG signals for operator clients | AI6=3: Behavioral/transaction data across 1,500+ operator brands is a useful proprietary set | AI7=3: Operators depend on its AI-enabled platform (anti-fraud, prediction markets) as infra | F1=4: Bootstrapped since 2009, scaled to 2,000+ staff without external funding | F2=3: Est. ~$420M revenue (unverified estimate); profitability not independently disclosed | F3=4: 15+ years bootstrapped operation; no runway/distress signals found | F4=None: Private company; leverage/debt terms not disclosed | F5=2: Privately held, no PE/VC backing or public listing found for capital access</t>
+        </is>
+      </c>
+      <c r="DJ26" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="DK26" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="DL26" t="inlineStr">
+        <is>
+          <t>sonnet/company-researcher</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Super Group (SGHC) Limited</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Guernsey (registered); international operations/tech hub in Malta and Bulgaria</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>2006</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Operator (B2C)</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Multi-brand operator uniting Betway (sportsbook) and Spin (casino); revenue from wagering margin, driven by heavy sports/esports sponsorship marketing rather than pure affiliate-SEO acquisition; NYSE-listed (SGHC) via 2023 SPAC merger with Digital Gaming Corp.</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>B2C sports bettors and casino players; core growth markets Africa (Nigeria, Ghana, South Africa), plus Europe, Canada and Latin America</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="Y27" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AA27" t="inlineStr">
+        <is>
+          <t>L0</t>
+        </is>
+      </c>
+      <c r="AC27" t="inlineStr">
+        <is>
+          <t>Large regulated African player base (Nigeria, Ghana, South Africa) — a differentiated data position versus Western-focused peers</t>
+        </is>
+      </c>
+      <c r="AF27" t="inlineStr">
+        <is>
+          <t>Large sports/esports sponsorship portfolio under Betway (incl. Aston Martin Aramco F1 Team, football clubs, ESL esports)</t>
+        </is>
+      </c>
+      <c r="AH27" t="inlineStr">
+        <is>
+          <t>Licensed across Africa (Nigeria, Ghana, South Africa et al.), multiple European markets, and Ontario, Canada; exited the UK online betting market in 2022</t>
+        </is>
+      </c>
+      <c r="AI27" t="n">
+        <v>100</v>
+      </c>
+      <c r="AL27" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AM27" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AN27" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AO27" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AP27" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AQ27" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AR27" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AS27" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AT27" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AV27" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AX27" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AZ27" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="BB27" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="BD27" t="n">
+        <v>3</v>
+      </c>
+      <c r="BI27" t="n">
+        <v>1</v>
+      </c>
+      <c r="BJ27" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK27" t="n">
+        <v>2</v>
+      </c>
+      <c r="BL27" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM27" t="n">
+        <v>2</v>
+      </c>
+      <c r="BN27" t="n">
+        <v>3</v>
+      </c>
+      <c r="BO27" t="n">
+        <v>4</v>
+      </c>
+      <c r="BP27" t="n">
+        <v>3</v>
+      </c>
+      <c r="BQ27" t="n">
+        <v>3</v>
+      </c>
+      <c r="BR27" t="n">
+        <v>4</v>
+      </c>
+      <c r="BS27" t="n">
+        <v>3</v>
+      </c>
+      <c r="BT27" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU27" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV27" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW27" t="n">
+        <v>1</v>
+      </c>
+      <c r="BX27" t="n">
+        <v>2</v>
+      </c>
+      <c r="BY27" t="n">
+        <v>3</v>
+      </c>
+      <c r="BZ27" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA27" t="n">
+        <v>22</v>
+      </c>
+      <c r="CB27" t="n">
+        <v>67</v>
+      </c>
+      <c r="CC27" t="n">
+        <v>15</v>
+      </c>
+      <c r="CD27" t="n">
+        <v>41</v>
+      </c>
+      <c r="CE27" t="n">
+        <v>33</v>
+      </c>
+      <c r="CF27" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="CG27" t="inlineStr">
+        <is>
+          <t>Dormant</t>
+        </is>
+      </c>
+      <c r="CH27" t="inlineStr">
+        <is>
+          <t>No AI assistant, prediction-market or direct-channel initiative found; still paid-marketing (sponsorship/affiliate) dependent for player acquisition.</t>
+        </is>
+      </c>
+      <c r="CJ27" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="CK27" t="inlineStr">
+        <is>
+          <t>3y+</t>
+        </is>
+      </c>
+      <c r="CL27" t="inlineStr">
+        <is>
+          <t>Standard multi-brand sponsorship/affiliate-acquired operator; reinforces the incumbent acquisition model rather than building an owned or AI-native player channel.</t>
+        </is>
+      </c>
+      <c r="CN27" t="inlineStr">
+        <is>
+          <t>Target was listed as 'Super Group (Betway) Limited'; resolved to the actual NYSE-listed legal entity Super Group (SGHC) Limited, of which Betway is the flagship sportsbook brand alongside the Spin casino brand. HQ/founding-year details carry medium confidence (Guernsey registration, Betway brand launch 2006) and should be re-verified against a 10-K/20-F filing if this company becomes decision-critical. Notably exited the UK online betting market in 2022 over affordability-check compliance costs — a real gap versus tier-1-market peers, reflected in D3.</t>
+        </is>
+      </c>
+      <c r="CQ27" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="CU27" t="inlineStr">
+        <is>
+          <t>Q1 2026 revenue $612m (+18% YoY), profit $86m, Adjusted EBITDA $152m (+36% YoY, 25% margin); FY2026 guidance revenue &gt;$2.55bn, Adjusted EBITDA &gt;$680m</t>
+        </is>
+      </c>
+      <c r="CY27" t="n">
+        <v>4</v>
+      </c>
+      <c r="CZ27" t="n">
+        <v>4</v>
+      </c>
+      <c r="DA27" t="n">
+        <v>5</v>
+      </c>
+      <c r="DC27" t="n">
+        <v>4</v>
+      </c>
+      <c r="DD27" t="n">
+        <v>85</v>
+      </c>
+      <c r="DE27" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="DH27" t="inlineStr">
+        <is>
+          <t>https://finance.yahoo.com/markets/stocks/articles/super-group-sghc-uses-betway-152946894.html ; https://www.gurufocus.com/news/8971626/super-group-to-report-second-quarter-2026-financial-results ; https://www.barchart.com/story/news/128311/super-group-to-report-fourth-quarter-and-full-year-2025-financial-results</t>
+        </is>
+      </c>
+      <c r="DI27" t="inlineStr">
+        <is>
+          <t>Resolved to Super Group (SGHC) Limited, NYSE-listed (ticker SGHC), parent of Betway (sportsbook) and Spin (casino) brands, formed via 2023 SPAC merger with Digital Gaming Corp. Q1 2026 results show strong growth (revenue $612m +18% YoY, Adjusted EBITDA $152m +36%) with FY2026 guidance raised to &gt;$2.55bn revenue / &gt;$680m Adjusted EBITDA. Reportable segments changed from Betway/Spin brands to Africa/International regions in Q1 2026, with Africa (notably a Nigeria push) now 44% of segment revenue ($267m). No AI-specific strategy, agentic capability, or commerce-protocol evidence surfaced in the searches run; AI scores reflect absence of found evidence rather than confirmed absence of capability. || W1=1: Standard operator marketing; no stance against affiliate/incumbent model | W2=1: Growth funded organically (Africa expansion); no AI/wallet M&amp;A found | W3=2: Large global sports/esports sponsorship portfolio, still brand marketing | W4=0: No AI assistant, wallet or prediction surface found shipped | W5=2: Sponsorship-driven brand awareness is paid, not truly owned intent | D1=3: Sportsbook + casino/live casino solid; poker/bingo not prominent | D2=4: Proprietary Betway sportsbook trading/risk management at scale | D3=3: Broad multi-market licensing, but notably exited UK in 2022 | D4=3: Licensed operator; payments via partners, owns player wallet | D5=4: Global reach (Africa/Europe/Canada/LatAm), $2.5bn+ FY26 revenue guide | D6=3: Betway globally recognized via sponsorship, solid but not top-tier trust | AI1=0: No evidence found of foundation-model use or development | AI2=0: No shipped agentic capability found | AI3=0: No MCP/A2A/UCP/ACP adoption evidence found | AI4=1: Likely only generic support chat; no differentiated assistant found | AI5=2: Company cites 'data-driven analytics' for engagement, unconfirmed depth | AI6=3: Large regulated African player base is a differentiated data set | AI7=0: No evidence of platform position in gen-AI ecosystem | F1=4: Profitable, growing, self-funding at scale (EBITDA guide &gt;$680m) | F2=4: Q1 2026: $612m revenue +18%, $86m profit, 25% EBITDA margin | F3=5: Public, profitable operator; no runway concern identified | F4=None: No confirmed leverage/debt figures found this pass | F5=4: NYSE-listed with public capital-markets access</t>
+        </is>
+      </c>
+      <c r="DJ27" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="DK27" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="DL27" t="inlineStr">
+        <is>
+          <t>sonnet/company-researcher</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Underdog Fantasy</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>New York, NY, US (medium confidence, not independently re-verified this session)</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>2020</v>
+      </c>
+      <c r="E28" t="n">
+        <v>115</v>
+      </c>
+      <c r="F28" t="n">
+        <v>1230</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>AI-native &amp; prediction markets</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Started as daily fantasy sports (Best Ball, Pick'em); expanded into a proprietary sportsbook (live in North Carolina, Mar 2024) and, since Sept 2025, sports/event prediction markets; acquired CFTC-registered exchange Aristotle (Mar 2026) to self-clear contracts. Revenue from contest entry fees (10-15%) and prediction-market spreads/fees. Agreed to be acquired by IG Group plc for up to ~$1.1-1.3bn (announced 30 Jul 2026, not yet closed).</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>B2C — US-based DFS players and sports bettors, now expanding into prediction-market traders across sports and non-sports categories (politics, crypto, culture, climate)</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="W28" t="inlineStr">
+        <is>
+          <t>Predictive/statistical optimization models for lineups and projections; no evidence of foundation-model (LLM) development</t>
+        </is>
+      </c>
+      <c r="Y28" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AA28" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="AC28" t="inlineStr">
+        <is>
+          <t>Millions of Best Ball/Pick'em entries plus prediction-market order flow across 25+ sports and non-sports categories</t>
+        </is>
+      </c>
+      <c r="AF28" t="inlineStr">
+        <is>
+          <t>Crypto.com (prediction-markets launch partner, Sept 2025, 16 states); pending acquisition by IG Group plc (agreed ~$1.1-1.3bn, announced 30 Jul 2026)</t>
+        </is>
+      </c>
+      <c r="AH28" t="inlineStr">
+        <is>
+          <t>DFS operating in 41 states + DC + Canada (ex-Ontario); sports-betting licenses in Ohio and Colorado with a live proprietary sportsbook in North Carolina; Aristotle Exchange is a CFTC-registered Designated Contract Market (DCM) and Derivatives Clearing Organization (DCO)</t>
+        </is>
+      </c>
+      <c r="AL28" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AM28" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AN28" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AO28" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AP28" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AQ28" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AR28" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AS28" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AT28" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AV28" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AX28" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AZ28" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="BB28" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="BD28" t="n">
+        <v>2</v>
+      </c>
+      <c r="BI28" t="n">
+        <v>5</v>
+      </c>
+      <c r="BJ28" t="n">
+        <v>4</v>
+      </c>
+      <c r="BK28" t="n">
+        <v>4</v>
+      </c>
+      <c r="BL28" t="n">
+        <v>5</v>
+      </c>
+      <c r="BM28" t="n">
+        <v>4</v>
+      </c>
+      <c r="BN28" t="n">
+        <v>4</v>
+      </c>
+      <c r="BO28" t="n">
+        <v>5</v>
+      </c>
+      <c r="BP28" t="n">
+        <v>5</v>
+      </c>
+      <c r="BQ28" t="n">
+        <v>3</v>
+      </c>
+      <c r="BR28" t="n">
+        <v>3</v>
+      </c>
+      <c r="BS28" t="n">
+        <v>4</v>
+      </c>
+      <c r="BT28" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU28" t="n">
+        <v>3</v>
+      </c>
+      <c r="BV28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW28" t="n">
+        <v>1</v>
+      </c>
+      <c r="BX28" t="n">
+        <v>4</v>
+      </c>
+      <c r="BY28" t="n">
+        <v>4</v>
+      </c>
+      <c r="BZ28" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA28" t="n">
+        <v>89</v>
+      </c>
+      <c r="CB28" t="n">
+        <v>83</v>
+      </c>
+      <c r="CC28" t="n">
+        <v>41</v>
+      </c>
+      <c r="CD28" t="n">
+        <v>62</v>
+      </c>
+      <c r="CE28" t="n">
+        <v>73</v>
+      </c>
+      <c r="CF28" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="CG28" t="inlineStr">
+        <is>
+          <t>Imminent threat</t>
+        </is>
+      </c>
+      <c r="CH28" t="inlineStr">
+        <is>
+          <t>Not yet at incumbent operator scale or global reach; no casino/live-casino/poker vertical; being folded into IG Group's public-markets structure via a pending, not-yet-closed acquisition.</t>
+        </is>
+      </c>
+      <c r="CJ28" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="CK28" t="inlineStr">
+        <is>
+          <t>0-12m</t>
+        </is>
+      </c>
+      <c r="CL28" t="inlineStr">
+        <is>
+          <t>A genuine three-pillar threat: organically-built owned audience, a shipped proprietary sportsbook plus prediction-market product, and real owned settlement/exchange infrastructure (Aristotle) — directly bypasses the licensed-operator/affiliate model the brief names as incumbent.</t>
+        </is>
+      </c>
+      <c r="CN28" t="inlineStr">
+        <is>
+          <t>Target name 'Underdog Fantasy' used as the operating brand; the precise US legal entity name was not independently re-verified this session (commonly referred to simply as 'Underdog' in 2026 press, reflecting its pivot beyond fantasy sports). The IG Group acquisition (announced ~30 Jul 2026, the day before this research) is AGREED, not yet confirmed closed — scores reflect Underdog's pre-close standalone trajectory, which is what drove IG's willingness to pay up to $1.3bn. Scored as the clear high-willingness outlier of this batch (W 88%), deliberately kept just below the Polymarket anchor (W 91%) since Polymarket's crypto-native, more frame-breaking positioning is still the willingness ceiling per anchors.md; Underdog remains a CFTC/state-regulated entity rather than a permissionless crypto-native platform. Distribution score (80%) is earned mainly by owning Aristotle Exchange (CFTC DCM/DCO) — genuine settlement infrastructure, not just a product feature — putting it well above typical AI-native/prediction-market startups (cf. Rithmm anchor, D 11%).</t>
+        </is>
+      </c>
+      <c r="CQ28" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="CU28" t="inlineStr">
+        <is>
+          <t>IG Group's pending acquisition is expected to more than double IG's US revenue and grow IG's US monthly-active-customer base 10x+ — implies substantial scale, though revenue is not independently disclosed; reached #3 US prediction-markets venue by regulated notional volume (behind only Kalshi and Robinhood) within months of its September 2025 launch</t>
+        </is>
+      </c>
+      <c r="CY28" t="n">
+        <v>4</v>
+      </c>
+      <c r="CZ28" t="n">
+        <v>3</v>
+      </c>
+      <c r="DA28" t="n">
+        <v>4</v>
+      </c>
+      <c r="DB28" t="n">
+        <v>4</v>
+      </c>
+      <c r="DC28" t="n">
+        <v>5</v>
+      </c>
+      <c r="DD28" t="n">
+        <v>80</v>
+      </c>
+      <c r="DE28" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="DH28" t="inlineStr">
+        <is>
+          <t>https://bettorsinsider.com/news/2026/07/31/ig-group-confirms-1-3-billion-acquisition-of-prediction-markets-operator-underdog/ ; https://www.sportspro.com/news/betting/underdog-fantasy-prediction-markets-aristotle-march-2026/ ; https://www.sportico.com/business/sports-betting/2026/underdog-prediction-market-aristotle-injury-updates-1234940046/ ; https://sacra.com/c/underdog-fantasy/</t>
+        </is>
+      </c>
+      <c r="DI28" t="inlineStr">
+        <is>
+          <t>Very fresh news: IG Group plc agreed on/around 30 Jul 2026 to acquire Underdog for up to $1.1-1.3bn, expected to more than double IG's US revenue and grow its US MAU base 10x+ — strong evidence Underdog has built real scale in prediction markets. Underdog entered event contracts via a Crypto.com partnership (Sept 2025, 16 states) and became the #3 US prediction-markets venue by regulated notional volume (behind Kalshi and Robinhood); its March 2026 acquisition of Aristotle Exchange (a CFTC-registered DCM and DCO) gave it a self-clearing, federally-regulated exchange — a rare and load-bearing distribution asset. Funding history (Sacra): $115M total raised, Series C (early 2025) valuing the company at ~$1.23bn, up from $485M in 2022; investors include BlackRock, Spark Capital, Acies Investment, Mark Cuban, Kevin Durant. Best Ball's automatic weekly lineup optimization is treated as a real shipped L2 agentic feature. || W1=5: Openly attacks the licensed operator model via prediction-market exchange | W2=4: Systematic reshaping: Aristotle acquisition, Crypto.com deal, Series C | W3=4: Crypto.com prediction-markets alliance; pending IG Group backing deal | W4=5: Fantasy + proprietary sportsbook + prediction markets + own exchange, all live | W5=4: Organically built #3 US prediction-market audience, not affiliate-bought | D1=4: Strong DFS/prediction-market content; no casino, live casino or poker | D2=5: Owns Aristotle Exchange (CFTC DCM/DCO) plus proprietary sportsbook tech | D3=5: State DFS/sportsbook licenses plus rare federal CFTC exchange registration | D4=3: Payments via Crypto.com and traditional PSP partners, not yet owned MoR | D5=3: Broad US-only reach (41 states+DC+Canada); #3 US venue by volume | D6=4: Elite-investor-backed, fast-growing trust in DFS/prediction-market niche | AI1=1: Statistical projection/optimization models, not foundation-model work | AI2=3: Best Ball auto-selects optimal weekly lineups without user input (L2) | AI3=0: No MCP/A2A/UCP/ACP adoption evidence found | AI4=1: No dedicated conversational assistant found beyond auto-lineup feature | AI5=4: Individual-level lineup/pick optimization is core to the product | AI6=4: Millions of entries plus prediction-market order flow across categories | AI7=0: Product/consumer company; no evidence others build on its AI/data | F1=4: $1.2B+ Series C plus pending $1.1-1.3B IG Group acquisition offer | F2=3: Implied substantial revenue via IG deal rationale; not independently confirmed | F3=4: Fresh mega-round plus pending strategic acquisition removes near-term risk | F4=4: Venture-equity funded; no debt/leverage signals found | F5=5: Elite investor base (BlackRock, Spark Capital, Mark Cuban) plus IG Group deal</t>
+        </is>
+      </c>
+      <c r="DJ28" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="DK28" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="DL28" t="inlineStr">
+        <is>
+          <t>sonnet/company-researcher</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>